<commit_message>
Header-based xlsx parsing with distant-month expiry; real leg quotes (bid/ask/IV) for open positions
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFpWXi6zDsMbHMMv6Bh7cj
</commit_message>
<xml_diff>
--- a/VTS_Iron_Condor_strategy.xlsx
+++ b/VTS_Iron_Condor_strategy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d0023b5393a4cbf7/文件/私人/Research/槓桿低波策略/Options/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{C33350A6-696F-0F44-BF9B-10BB1A4F9F32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40D7D106-E281-4239-9A6D-0AD9D8F90FF1}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{B52C6A47-3491-41B8-A7C0-A1EF4207AA0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A78A769-F22E-40A7-AACE-6114C47962D2}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{E5885415-119C-814A-8DF0-43BBE85569FC}"/>
+    <workbookView xWindow="15" yWindow="15" windowWidth="21585" windowHeight="13665" xr2:uid="{E5885415-119C-814A-8DF0-43BBE85569FC}"/>
   </bookViews>
   <sheets>
     <sheet name="IB Option Paper Trade" sheetId="2" r:id="rId1"/>
@@ -784,7 +784,22 @@
         </r>
       </text>
     </comment>
-    <comment ref="I7" authorId="0" shapeId="0" xr:uid="{4CD305E1-C860-4714-94C0-F4A5D9ABF60E}">
+    <comment ref="I7" authorId="0" shapeId="0" xr:uid="{8B05A1EA-E43A-4526-8DD4-3F3BE83C4525}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>The expiration date for the distant-month contract (only for Calendars).
+Leave the space for Iron Condors.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J7" authorId="0" shapeId="0" xr:uid="{4CD305E1-C860-4714-94C0-F4A5D9ABF60E}">
       <text>
         <r>
           <rPr>
@@ -831,7 +846,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J7" authorId="0" shapeId="0" xr:uid="{34C28669-750D-481D-A3B0-2518CC8F74B6}">
+    <comment ref="K7" authorId="0" shapeId="0" xr:uid="{34C28669-750D-481D-A3B0-2518CC8F74B6}">
       <text>
         <r>
           <rPr>
@@ -845,7 +860,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K7" authorId="0" shapeId="0" xr:uid="{4C993F10-0A8B-42C1-9684-52DE0C122C94}">
+    <comment ref="L7" authorId="0" shapeId="0" xr:uid="{4C993F10-0A8B-42C1-9684-52DE0C122C94}">
       <text>
         <r>
           <rPr>
@@ -892,7 +907,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L7" authorId="0" shapeId="0" xr:uid="{81C004A5-13A7-4212-B764-90F3B8FCB433}">
+    <comment ref="M7" authorId="0" shapeId="0" xr:uid="{81C004A5-13A7-4212-B764-90F3B8FCB433}">
       <text>
         <r>
           <rPr>
@@ -928,7 +943,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M7" authorId="0" shapeId="0" xr:uid="{82BCD69D-1E28-41A3-97B7-6E97ED99762B}">
+    <comment ref="N7" authorId="0" shapeId="0" xr:uid="{82BCD69D-1E28-41A3-97B7-6E97ED99762B}">
       <text>
         <r>
           <rPr>
@@ -964,7 +979,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N7" authorId="0" shapeId="0" xr:uid="{A659FF58-2675-42B4-989A-F4AED97BA17D}">
+    <comment ref="O7" authorId="0" shapeId="0" xr:uid="{A659FF58-2675-42B4-989A-F4AED97BA17D}">
       <text>
         <r>
           <rPr>
@@ -1000,7 +1015,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O7" authorId="0" shapeId="0" xr:uid="{4FA46A78-3C2E-4310-8D5F-FEFC550EF977}">
+    <comment ref="P7" authorId="0" shapeId="0" xr:uid="{4FA46A78-3C2E-4310-8D5F-FEFC550EF977}">
       <text>
         <r>
           <rPr>
@@ -1036,7 +1051,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P7" authorId="0" shapeId="0" xr:uid="{EE6036B4-05BC-49CE-A677-CCACD17C33B1}">
+    <comment ref="Q7" authorId="0" shapeId="0" xr:uid="{EE6036B4-05BC-49CE-A677-CCACD17C33B1}">
       <text>
         <r>
           <rPr>
@@ -1072,7 +1087,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q7" authorId="0" shapeId="0" xr:uid="{0DD1D602-F7D1-4F43-911D-67D07B9934A3}">
+    <comment ref="R7" authorId="0" shapeId="0" xr:uid="{0DD1D602-F7D1-4F43-911D-67D07B9934A3}">
       <text>
         <r>
           <rPr>
@@ -1108,7 +1123,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R7" authorId="0" shapeId="0" xr:uid="{EC68FE36-4D56-4219-88DE-7A57D74D2FD3}">
+    <comment ref="S7" authorId="0" shapeId="0" xr:uid="{EC68FE36-4D56-4219-88DE-7A57D74D2FD3}">
       <text>
         <r>
           <rPr>
@@ -1144,7 +1159,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S7" authorId="0" shapeId="0" xr:uid="{AB1C05BC-7875-476C-989B-B33BCC88B515}">
+    <comment ref="T7" authorId="0" shapeId="0" xr:uid="{AB1C05BC-7875-476C-989B-B33BCC88B515}">
       <text>
         <r>
           <rPr>
@@ -1191,7 +1206,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T7" authorId="0" shapeId="0" xr:uid="{712A1EBC-87A4-42C2-AC05-1B9C1B9D2DB8}">
+    <comment ref="U7" authorId="0" shapeId="0" xr:uid="{712A1EBC-87A4-42C2-AC05-1B9C1B9D2DB8}">
       <text>
         <r>
           <rPr>
@@ -1238,7 +1253,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="U7" authorId="0" shapeId="0" xr:uid="{6DC21F5F-F484-48DF-8615-D5B129541065}">
+    <comment ref="V7" authorId="0" shapeId="0" xr:uid="{6DC21F5F-F484-48DF-8615-D5B129541065}">
       <text>
         <r>
           <rPr>
@@ -1285,7 +1300,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="V7" authorId="0" shapeId="0" xr:uid="{831B29CA-EFC3-4503-A853-3FBE63F1AFE5}">
+    <comment ref="W7" authorId="0" shapeId="0" xr:uid="{831B29CA-EFC3-4503-A853-3FBE63F1AFE5}">
       <text>
         <r>
           <rPr>
@@ -1332,7 +1347,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="W7" authorId="0" shapeId="0" xr:uid="{E9564960-4D5D-4C9D-8BEE-CF5D7DC06F0D}">
+    <comment ref="X7" authorId="0" shapeId="0" xr:uid="{E9564960-4D5D-4C9D-8BEE-CF5D7DC06F0D}">
       <text>
         <r>
           <rPr>
@@ -1368,7 +1383,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="X7" authorId="0" shapeId="0" xr:uid="{75A82223-A2E5-4696-A1C0-18AB9ABE1084}">
+    <comment ref="Y7" authorId="0" shapeId="0" xr:uid="{75A82223-A2E5-4696-A1C0-18AB9ABE1084}">
       <text>
         <r>
           <rPr>
@@ -1415,7 +1430,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Y7" authorId="0" shapeId="0" xr:uid="{369CA303-B93F-4574-BD0D-B82C35B00447}">
+    <comment ref="Z7" authorId="0" shapeId="0" xr:uid="{369CA303-B93F-4574-BD0D-B82C35B00447}">
       <text>
         <r>
           <rPr>
@@ -1452,7 +1467,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z7" authorId="0" shapeId="0" xr:uid="{4627D1AE-CE73-49BE-802C-3906B9F5C664}">
+    <comment ref="AA7" authorId="0" shapeId="0" xr:uid="{4627D1AE-CE73-49BE-802C-3906B9F5C664}">
       <text>
         <r>
           <rPr>
@@ -1488,7 +1503,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AA7" authorId="0" shapeId="0" xr:uid="{C5B2A55B-EB20-45A7-9B1C-475D8B9E840D}">
+    <comment ref="AB7" authorId="0" shapeId="0" xr:uid="{C5B2A55B-EB20-45A7-9B1C-475D8B9E840D}">
       <text>
         <r>
           <rPr>
@@ -1524,7 +1539,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB7" authorId="0" shapeId="0" xr:uid="{5664355A-D057-4DDD-8347-73EB8DAC7F1E}">
+    <comment ref="AC7" authorId="0" shapeId="0" xr:uid="{5664355A-D057-4DDD-8347-73EB8DAC7F1E}">
       <text>
         <r>
           <rPr>
@@ -1560,7 +1575,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AC7" authorId="0" shapeId="0" xr:uid="{9E70E910-B8E8-441A-A7CB-BE87505697FF}">
+    <comment ref="AD7" authorId="0" shapeId="0" xr:uid="{9E70E910-B8E8-441A-A7CB-BE87505697FF}">
       <text>
         <r>
           <rPr>
@@ -1596,7 +1611,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AD7" authorId="0" shapeId="0" xr:uid="{8F3AEC79-3EF4-4B73-B239-763914DC86B3}">
+    <comment ref="AE7" authorId="0" shapeId="0" xr:uid="{8F3AEC79-3EF4-4B73-B239-763914DC86B3}">
       <text>
         <r>
           <rPr>
@@ -1632,7 +1647,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AE7" authorId="0" shapeId="0" xr:uid="{F14F30D5-D8C3-4AF1-AADC-B28309AF0AFB}">
+    <comment ref="AF7" authorId="0" shapeId="0" xr:uid="{F14F30D5-D8C3-4AF1-AADC-B28309AF0AFB}">
       <text>
         <r>
           <rPr>
@@ -1668,7 +1683,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AF7" authorId="0" shapeId="0" xr:uid="{AEA0F864-CF79-4D84-AD45-B229567C340A}">
+    <comment ref="AG7" authorId="0" shapeId="0" xr:uid="{AEA0F864-CF79-4D84-AD45-B229567C340A}">
       <text>
         <r>
           <rPr>
@@ -1704,7 +1719,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AH7" authorId="0" shapeId="0" xr:uid="{B68832D3-B4E6-4087-9BCA-83A25E6B3CD8}">
+    <comment ref="AI7" authorId="0" shapeId="0" xr:uid="{B68832D3-B4E6-4087-9BCA-83A25E6B3CD8}">
       <text>
         <r>
           <rPr>
@@ -1727,7 +1742,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AI7" authorId="0" shapeId="0" xr:uid="{1B313849-A0F7-464E-B52E-954F02A52FB0}">
+    <comment ref="AJ7" authorId="0" shapeId="0" xr:uid="{1B313849-A0F7-464E-B52E-954F02A52FB0}">
       <text>
         <r>
           <rPr>
@@ -1741,7 +1756,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AJ7" authorId="1" shapeId="0" xr:uid="{5E34C5CD-2397-4916-9FD7-3E06DD5EEF01}">
+    <comment ref="AK7" authorId="1" shapeId="0" xr:uid="{5E34C5CD-2397-4916-9FD7-3E06DD5EEF01}">
       <text>
         <r>
           <rPr>
@@ -1755,7 +1770,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AK7" authorId="0" shapeId="0" xr:uid="{31D402E3-E4A0-4F3C-92C8-418185773AAE}">
+    <comment ref="AL7" authorId="0" shapeId="0" xr:uid="{31D402E3-E4A0-4F3C-92C8-418185773AAE}">
       <text>
         <r>
           <rPr>
@@ -1769,7 +1784,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AL7" authorId="0" shapeId="0" xr:uid="{5317E72C-4AF4-4937-AE5A-BCCE1B7B87BC}">
+    <comment ref="AM7" authorId="0" shapeId="0" xr:uid="{5317E72C-4AF4-4937-AE5A-BCCE1B7B87BC}">
       <text>
         <r>
           <rPr>
@@ -1783,7 +1798,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AM7" authorId="0" shapeId="0" xr:uid="{ACEE86E5-682F-471C-8DA1-81FEB558DDC4}">
+    <comment ref="AN7" authorId="0" shapeId="0" xr:uid="{ACEE86E5-682F-471C-8DA1-81FEB558DDC4}">
       <text>
         <r>
           <rPr>
@@ -1830,7 +1845,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AN7" authorId="0" shapeId="0" xr:uid="{70D47F45-19E8-4CBC-A7FF-146A749F1076}">
+    <comment ref="AO7" authorId="0" shapeId="0" xr:uid="{70D47F45-19E8-4CBC-A7FF-146A749F1076}">
       <text>
         <r>
           <rPr>
@@ -1877,7 +1892,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AO7" authorId="0" shapeId="0" xr:uid="{DDD669B4-6543-4BDD-9DD4-6D2D2A0CDD40}">
+    <comment ref="AP7" authorId="0" shapeId="0" xr:uid="{DDD669B4-6543-4BDD-9DD4-6D2D2A0CDD40}">
       <text>
         <r>
           <rPr>
@@ -1891,7 +1906,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AP7" authorId="0" shapeId="0" xr:uid="{F36C1074-E809-46AD-89FC-D87416B6E545}">
+    <comment ref="AQ7" authorId="0" shapeId="0" xr:uid="{F36C1074-E809-46AD-89FC-D87416B6E545}">
       <text>
         <r>
           <rPr>
@@ -1938,7 +1953,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AQ7" authorId="1" shapeId="0" xr:uid="{5B33410A-9288-4277-B2F2-BE7F0F65CE99}">
+    <comment ref="AR7" authorId="1" shapeId="0" xr:uid="{5B33410A-9288-4277-B2F2-BE7F0F65CE99}">
       <text>
         <r>
           <rPr>
@@ -1974,7 +1989,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AR7" authorId="0" shapeId="0" xr:uid="{1571A70A-B78B-4FC9-A485-2019B8597AC4}">
+    <comment ref="AS7" authorId="0" shapeId="0" xr:uid="{1571A70A-B78B-4FC9-A485-2019B8597AC4}">
       <text>
         <r>
           <rPr>
@@ -2021,7 +2036,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AS7" authorId="0" shapeId="0" xr:uid="{144F7BC4-2D6B-40FC-8D51-B9C17BE5CCBF}">
+    <comment ref="AT7" authorId="0" shapeId="0" xr:uid="{144F7BC4-2D6B-40FC-8D51-B9C17BE5CCBF}">
       <text>
         <r>
           <rPr>
@@ -4122,7 +4137,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="54">
   <si>
     <t>Strategy details</t>
   </si>
@@ -4278,6 +4293,16 @@
   </si>
   <si>
     <t>SPY</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>Expiration date
+(Near-month)</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>Expiration date
+(Distant-month)</t>
     <phoneticPr fontId="9" type="noConversion"/>
   </si>
 </sst>
@@ -4849,28 +4874,31 @@
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
-  <dimension ref="A2:AS33"/>
+  <dimension ref="A2:AT33"/>
   <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="5" width="20.796875" style="2" customWidth="1"/>
     <col min="6" max="6" width="20.796875" style="3" customWidth="1"/>
-    <col min="7" max="9" width="20.796875" style="2" customWidth="1"/>
-    <col min="10" max="10" width="20.796875" style="4" customWidth="1"/>
-    <col min="11" max="12" width="20.796875" style="2" customWidth="1"/>
-    <col min="13" max="14" width="20.796875" style="4" customWidth="1"/>
-    <col min="15" max="44" width="20.796875" style="2" customWidth="1"/>
-    <col min="45" max="45" width="166.6640625" style="2" customWidth="1"/>
-    <col min="46" max="139" width="20.796875" style="2" customWidth="1"/>
-    <col min="140" max="16384" width="10.796875" style="2"/>
+    <col min="7" max="7" width="20.796875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="22.73046875" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.73046875" style="2" customWidth="1"/>
+    <col min="10" max="10" width="20.796875" style="2" customWidth="1"/>
+    <col min="11" max="11" width="20.796875" style="4" customWidth="1"/>
+    <col min="12" max="13" width="20.796875" style="2" customWidth="1"/>
+    <col min="14" max="15" width="20.796875" style="4" customWidth="1"/>
+    <col min="16" max="45" width="20.796875" style="2" customWidth="1"/>
+    <col min="46" max="46" width="166.6640625" style="2" customWidth="1"/>
+    <col min="47" max="140" width="20.796875" style="2" customWidth="1"/>
+    <col min="141" max="16384" width="10.796875" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5"/>
-    <row r="4" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5"/>
+    <row r="4" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A4" s="5"/>
       <c r="B4" s="6" t="s">
         <v>1</v>
@@ -4883,109 +4911,110 @@
       </c>
       <c r="G4" s="9"/>
       <c r="H4" s="7"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="11"/>
-      <c r="K4" s="12"/>
-      <c r="L4" s="13"/>
-      <c r="M4" s="14" t="s">
-        <v>2</v>
-      </c>
+      <c r="I4" s="7"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="11"/>
+      <c r="L4" s="12"/>
+      <c r="M4" s="13"/>
       <c r="N4" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="O4" s="9"/>
+      <c r="O4" s="14" t="s">
+        <v>2</v>
+      </c>
       <c r="P4" s="9"/>
       <c r="Q4" s="9"/>
       <c r="R4" s="9"/>
       <c r="S4" s="9"/>
-      <c r="T4" s="5"/>
-      <c r="U4" s="15">
-        <f>((R4-Q4)-S4)*(T4*100)</f>
+      <c r="T4" s="9"/>
+      <c r="U4" s="5"/>
+      <c r="V4" s="15">
+        <f>((S4-R4)-T4)*(U4*100)</f>
         <v>0</v>
       </c>
-      <c r="V4" s="15">
+      <c r="W4" s="15">
         <f>E4*0.03</f>
         <v>0</v>
       </c>
-      <c r="W4" s="15">
-        <f>(R4-Q4)</f>
+      <c r="X4" s="15">
+        <f>(S4-R4)</f>
         <v>0</v>
       </c>
-      <c r="X4" s="16" t="e">
-        <f>(W4-S4)/W4</f>
-        <v>#DIV/0!</v>
-      </c>
       <c r="Y4" s="16" t="e">
-        <f>(P4-G4)/G4</f>
+        <f>(X4-T4)/X4</f>
         <v>#DIV/0!</v>
       </c>
       <c r="Z4" s="16" t="e">
         <f>(Q4-G4)/G4</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AA4" s="15">
-        <f>S4*0.5</f>
+      <c r="AA4" s="16" t="e">
+        <f>(R4-G4)/G4</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AB4" s="15">
+        <f>T4*0.5</f>
         <v>0</v>
       </c>
-      <c r="AB4" s="15">
-        <f>(S4*0.5)*(T4*100)</f>
+      <c r="AC4" s="15">
+        <f>(T4*0.5)*(U4*100)</f>
         <v>0</v>
       </c>
-      <c r="AC4" s="17">
-        <f>S4*1.5</f>
+      <c r="AD4" s="17">
+        <f>T4*1.5</f>
         <v>0</v>
       </c>
-      <c r="AD4" s="17">
-        <f>-((S4/2)*(T4*100))</f>
+      <c r="AE4" s="17">
+        <f>-((T4/2)*(U4*100))</f>
         <v>0</v>
       </c>
-      <c r="AE4" s="15">
+      <c r="AF4" s="15">
         <f>G4*0.96</f>
         <v>0</v>
       </c>
-      <c r="AF4" s="15">
+      <c r="AG4" s="15">
         <f>G4*1.04</f>
         <v>0</v>
       </c>
-      <c r="AG4" s="18"/>
-      <c r="AH4" s="7"/>
-      <c r="AI4" s="9"/>
-      <c r="AJ4" s="16" t="e">
-        <f>(AI4-G4)/G4</f>
+      <c r="AH4" s="18"/>
+      <c r="AI4" s="7"/>
+      <c r="AJ4" s="9"/>
+      <c r="AK4" s="16" t="e">
+        <f>(AJ4-G4)/G4</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AK4" s="9"/>
-      <c r="AL4" s="6">
-        <f>AH4-C4</f>
+      <c r="AL4" s="9"/>
+      <c r="AM4" s="6">
+        <f>AI4-C4</f>
         <v>0</v>
       </c>
-      <c r="AM4" s="15">
-        <f>((T4*4)*2)*0.65</f>
+      <c r="AN4" s="15">
+        <f>((U4*4)*2)*0.65</f>
         <v>0</v>
       </c>
-      <c r="AN4" s="16" t="e">
-        <f>AM4/U4</f>
+      <c r="AO4" s="16" t="e">
+        <f>AN4/V4</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AO4" s="15">
-        <f>((S4-AK4)*(T4*100))-AM4</f>
+      <c r="AP4" s="15">
+        <f>((T4-AL4)*(U4*100))-AN4</f>
         <v>0</v>
       </c>
-      <c r="AP4" s="16" t="e">
-        <f>AO4/U4</f>
+      <c r="AQ4" s="16" t="e">
+        <f>AP4/V4</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AQ4" s="26" t="e">
-        <f>AO4/(E4*0.2)</f>
+      <c r="AR4" s="26" t="e">
+        <f>AP4/(E4*0.2)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AR4" s="16" t="e">
-        <f>AO4/E4</f>
+      <c r="AS4" s="16" t="e">
+        <f>AP4/E4</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS4" s="8"/>
+      <c r="AT4" s="8"/>
     </row>
-    <row r="5" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A5" s="5"/>
       <c r="B5" s="6" t="s">
         <v>3</v>
@@ -4998,111 +5027,112 @@
       </c>
       <c r="G5" s="9"/>
       <c r="H5" s="7"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="12"/>
-      <c r="L5" s="13"/>
-      <c r="M5" s="14" t="s">
-        <v>4</v>
-      </c>
+      <c r="I5" s="7"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="11"/>
+      <c r="L5" s="12"/>
+      <c r="M5" s="13"/>
       <c r="N5" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="O5" s="9"/>
+      <c r="O5" s="14" t="s">
+        <v>4</v>
+      </c>
       <c r="P5" s="9"/>
-      <c r="Q5" s="15" t="s">
-        <v>4</v>
-      </c>
+      <c r="Q5" s="9"/>
       <c r="R5" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="S5" s="9"/>
-      <c r="T5" s="5"/>
-      <c r="U5" s="15">
-        <f>S5*(T5*100)</f>
+      <c r="S5" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="T5" s="9"/>
+      <c r="U5" s="5"/>
+      <c r="V5" s="15">
+        <f>T5*(U5*100)</f>
         <v>0</v>
       </c>
-      <c r="V5" s="15">
+      <c r="W5" s="15">
         <f>E5*0.02</f>
         <v>0</v>
       </c>
-      <c r="W5" s="15" t="s">
+      <c r="X5" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="X5" s="16" t="s">
+      <c r="Y5" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="Y5" s="16" t="e">
-        <f>(G5-P5)/G5</f>
+      <c r="Z5" s="16" t="e">
+        <f>(G5-Q5)/G5</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="Z5" s="16" t="s">
+      <c r="AA5" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="AA5" s="15">
-        <f>S5*1.25</f>
+      <c r="AB5" s="15">
+        <f>T5*1.25</f>
         <v>0</v>
       </c>
-      <c r="AB5" s="15">
-        <f>(S5*0.25)*(T5*100)</f>
+      <c r="AC5" s="15">
+        <f>(T5*0.25)*(U5*100)</f>
         <v>0</v>
       </c>
-      <c r="AC5" s="17">
-        <f>S5*0.75</f>
+      <c r="AD5" s="17">
+        <f>T5*0.75</f>
         <v>0</v>
       </c>
-      <c r="AD5" s="17">
-        <f>-((S5*0.25)*(T5*100))</f>
+      <c r="AE5" s="17">
+        <f>-((T5*0.25)*(U5*100))</f>
         <v>0</v>
       </c>
-      <c r="AE5" s="15">
+      <c r="AF5" s="15">
         <f>G5*0.96</f>
         <v>0</v>
       </c>
-      <c r="AF5" s="15">
+      <c r="AG5" s="15">
         <f>G5*1.04</f>
         <v>0</v>
       </c>
-      <c r="AG5" s="18"/>
-      <c r="AH5" s="7"/>
-      <c r="AI5" s="9"/>
-      <c r="AJ5" s="16" t="e">
-        <f>(AI5-G5)/G5</f>
+      <c r="AH5" s="18"/>
+      <c r="AI5" s="7"/>
+      <c r="AJ5" s="9"/>
+      <c r="AK5" s="16" t="e">
+        <f>(AJ5-G5)/G5</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AK5" s="9"/>
-      <c r="AL5" s="6">
-        <f>AH5-C5</f>
+      <c r="AL5" s="9"/>
+      <c r="AM5" s="6">
+        <f>AI5-C5</f>
         <v>0</v>
       </c>
-      <c r="AM5" s="15">
-        <f>((T5*2)*2)*0.65</f>
+      <c r="AN5" s="15">
+        <f>((U5*2)*2)*0.65</f>
         <v>0</v>
       </c>
-      <c r="AN5" s="16" t="e">
-        <f>AM5/U5</f>
+      <c r="AO5" s="16" t="e">
+        <f>AN5/V5</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AO5" s="15">
-        <f>((AK5-S5)*(T5*100))-AM5</f>
+      <c r="AP5" s="15">
+        <f>((AL5-T5)*(U5*100))-AN5</f>
         <v>0</v>
       </c>
-      <c r="AP5" s="16" t="e">
-        <f>AO5/U5</f>
+      <c r="AQ5" s="16" t="e">
+        <f>AP5/V5</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AQ5" s="26" t="e">
-        <f>AO5/(E5*0.2)</f>
+      <c r="AR5" s="26" t="e">
+        <f>AP5/(E5*0.2)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AR5" s="16" t="e">
-        <f>AO5/E5</f>
+      <c r="AS5" s="16" t="e">
+        <f>AP5/E5</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS5" s="8"/>
+      <c r="AT5" s="8"/>
     </row>
-    <row r="6" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5"/>
-    <row r="7" spans="1:45" ht="50" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5"/>
+    <row r="7" spans="1:46" ht="50" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A7" s="19" t="s">
         <v>5</v>
       </c>
@@ -5125,120 +5155,123 @@
         <v>11</v>
       </c>
       <c r="H7" s="19" t="s">
-        <v>12</v>
+        <v>52</v>
       </c>
       <c r="I7" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="J7" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="J7" s="21" t="s">
+      <c r="K7" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="K7" s="12" t="s">
+      <c r="L7" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="L7" s="21" t="s">
+      <c r="M7" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="M7" s="15" t="s">
+      <c r="N7" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="N7" s="15" t="s">
+      <c r="O7" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="O7" s="8" t="s">
+      <c r="P7" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="P7" s="22" t="s">
+      <c r="Q7" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="Q7" s="8" t="s">
+      <c r="R7" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="R7" s="8" t="s">
+      <c r="S7" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="S7" s="19" t="s">
+      <c r="T7" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="T7" s="19" t="s">
+      <c r="U7" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="U7" s="20" t="s">
+      <c r="V7" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="V7" s="20" t="s">
+      <c r="W7" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="W7" s="23" t="s">
+      <c r="X7" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="X7" s="24" t="s">
+      <c r="Y7" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="Y7" s="24" t="s">
+      <c r="Z7" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="Z7" s="24" t="s">
+      <c r="AA7" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="AA7" s="20" t="s">
+      <c r="AB7" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="AB7" s="20" t="s">
+      <c r="AC7" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="AC7" s="20" t="s">
+      <c r="AD7" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="AD7" s="20" t="s">
+      <c r="AE7" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="AE7" s="24" t="s">
+      <c r="AF7" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="AF7" s="24" t="s">
+      <c r="AG7" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="AG7" s="18"/>
-      <c r="AH7" s="8" t="s">
+      <c r="AH7" s="18"/>
+      <c r="AI7" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="AI7" s="8" t="s">
+      <c r="AJ7" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="AJ7" s="24" t="s">
+      <c r="AK7" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="AK7" s="8" t="s">
+      <c r="AL7" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="AL7" s="24" t="s">
+      <c r="AM7" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="AM7" s="24" t="s">
+      <c r="AN7" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="AN7" s="24" t="s">
+      <c r="AO7" s="24" t="s">
         <v>42</v>
       </c>
-      <c r="AO7" s="24" t="s">
+      <c r="AP7" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="AP7" s="24" t="s">
+      <c r="AQ7" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="AQ7" s="27" t="s">
+      <c r="AR7" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="AR7" s="24" t="s">
+      <c r="AS7" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="AS7" s="8" t="s">
+      <c r="AT7" s="8" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="8" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5"/>
-    <row r="9" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5"/>
+    <row r="9" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A9" s="30"/>
       <c r="B9" s="6" t="s">
         <v>3</v>
@@ -5261,132 +5294,135 @@
       <c r="H9" s="7">
         <v>46283</v>
       </c>
-      <c r="I9" s="5">
+      <c r="I9" s="7">
+        <v>46311</v>
+      </c>
+      <c r="J9" s="5">
         <v>22</v>
       </c>
-      <c r="J9" s="11">
+      <c r="K9" s="11">
         <v>14.51</v>
       </c>
-      <c r="K9" s="28">
+      <c r="L9" s="28">
         <v>0.05</v>
       </c>
-      <c r="L9" s="13">
+      <c r="M9" s="13">
         <v>0.14399999999999999</v>
-      </c>
-      <c r="M9" s="14" t="s">
-        <v>4</v>
       </c>
       <c r="N9" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="O9" s="9">
-        <v>770</v>
+      <c r="O9" s="14" t="s">
+        <v>4</v>
       </c>
       <c r="P9" s="9">
         <v>770</v>
       </c>
-      <c r="Q9" s="15" t="s">
-        <v>4</v>
+      <c r="Q9" s="9">
+        <v>770</v>
       </c>
       <c r="R9" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="S9" s="9">
+      <c r="S9" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="T9" s="9">
         <v>4.9400000000000004</v>
       </c>
-      <c r="T9" s="5">
+      <c r="U9" s="5">
         <v>46</v>
       </c>
-      <c r="U9" s="15">
-        <f>S9*(T9*100)</f>
+      <c r="V9" s="15">
+        <f>T9*(U9*100)</f>
         <v>22724</v>
       </c>
-      <c r="V9" s="15">
+      <c r="W9" s="15">
         <f>E9*0.02</f>
         <v>23011.336000000003</v>
       </c>
-      <c r="W9" s="15" t="s">
+      <c r="X9" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="X9" s="16" t="s">
+      <c r="Y9" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="Y9" s="16">
-        <f>(G9-P9)/G9</f>
+      <c r="Z9" s="16">
+        <f>(G9-Q9)/G9</f>
         <v>4.2838783378557359E-4</v>
       </c>
-      <c r="Z9" s="16" t="s">
+      <c r="AA9" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="AA9" s="15">
-        <f>S9*1.25</f>
+      <c r="AB9" s="15">
+        <f>T9*1.25</f>
         <v>6.1750000000000007</v>
       </c>
-      <c r="AB9" s="15">
-        <f>(S9*0.25)*(T9*100)</f>
+      <c r="AC9" s="15">
+        <f>(T9*0.25)*(U9*100)</f>
         <v>5681</v>
       </c>
-      <c r="AC9" s="17">
-        <f>S9*0.75</f>
+      <c r="AD9" s="17">
+        <f>T9*0.75</f>
         <v>3.7050000000000001</v>
       </c>
-      <c r="AD9" s="17">
-        <f>-((S9*0.25)*(T9*100))</f>
+      <c r="AE9" s="17">
+        <f>-((T9*0.25)*(U9*100))</f>
         <v>-5681</v>
       </c>
-      <c r="AE9" s="15">
+      <c r="AF9" s="15">
         <f>G9*0.96</f>
         <v>739.51679999999999</v>
       </c>
-      <c r="AF9" s="15">
+      <c r="AG9" s="15">
         <f>G9*1.04</f>
         <v>801.14320000000009</v>
       </c>
-      <c r="AG9" s="18"/>
-      <c r="AH9" s="7">
+      <c r="AH9" s="18"/>
+      <c r="AI9" s="7">
         <v>46281</v>
       </c>
-      <c r="AI9" s="9">
+      <c r="AJ9" s="9">
         <v>754.05</v>
       </c>
-      <c r="AJ9" s="16">
-        <f>(AI9-G9)/G9</f>
+      <c r="AK9" s="16">
+        <f>(AJ9-G9)/G9</f>
         <v>-2.1133799800085788E-2</v>
       </c>
-      <c r="AK9" s="9">
+      <c r="AL9" s="9">
         <v>3.8</v>
       </c>
-      <c r="AL9" s="6">
-        <f>AH9-C9</f>
+      <c r="AM9" s="6">
+        <f>AI9-C9</f>
         <v>20</v>
       </c>
-      <c r="AM9" s="15">
-        <f>((T9*2)*2)*0.65</f>
+      <c r="AN9" s="15">
+        <f>((U9*2)*2)*0.65</f>
         <v>119.60000000000001</v>
       </c>
-      <c r="AN9" s="16">
-        <f>AM9/U9</f>
+      <c r="AO9" s="16">
+        <f>AN9/V9</f>
         <v>5.2631578947368429E-3</v>
       </c>
-      <c r="AO9" s="15">
-        <f>((AK9-S9)*(T9*100))-AM9</f>
+      <c r="AP9" s="15">
+        <f>((AL9-T9)*(U9*100))-AN9</f>
         <v>-5363.6000000000031</v>
       </c>
-      <c r="AP9" s="16">
-        <f>AO9/U9</f>
+      <c r="AQ9" s="16">
+        <f>AP9/V9</f>
         <v>-0.23603238866396775</v>
       </c>
-      <c r="AQ9" s="26">
-        <f>AO9/(E9*0.2)</f>
+      <c r="AR9" s="26">
+        <f>AP9/(E9*0.2)</f>
         <v>-2.3308511943852382E-2</v>
       </c>
-      <c r="AR9" s="16">
-        <f>AO9/E9</f>
+      <c r="AS9" s="16">
+        <f>AP9/E9</f>
         <v>-4.6617023887704761E-3</v>
       </c>
-      <c r="AS9" s="8"/>
+      <c r="AT9" s="8"/>
     </row>
-    <row r="10" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A10" s="29"/>
       <c r="B10" s="6" t="s">
         <v>3</v>
@@ -5409,126 +5445,129 @@
       <c r="H10" s="7">
         <v>46346</v>
       </c>
-      <c r="I10" s="5">
+      <c r="I10" s="7">
+        <v>46374</v>
+      </c>
+      <c r="J10" s="5">
         <v>51</v>
       </c>
-      <c r="J10" s="11">
+      <c r="K10" s="11">
         <v>15.77</v>
       </c>
-      <c r="K10" s="12">
+      <c r="L10" s="12">
         <v>0.28000000000000003</v>
       </c>
-      <c r="L10" s="13">
+      <c r="M10" s="13">
         <v>0.37559999999999999</v>
-      </c>
-      <c r="M10" s="14" t="s">
-        <v>4</v>
       </c>
       <c r="N10" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="O10" s="9">
-        <v>768</v>
+      <c r="O10" s="14" t="s">
+        <v>4</v>
       </c>
       <c r="P10" s="9">
         <v>768</v>
       </c>
-      <c r="Q10" s="15" t="s">
-        <v>4</v>
+      <c r="Q10" s="9">
+        <v>768</v>
       </c>
       <c r="R10" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="S10" s="9">
+      <c r="S10" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="T10" s="9">
         <v>3.78</v>
       </c>
-      <c r="T10" s="5">
+      <c r="U10" s="5">
         <v>60</v>
       </c>
-      <c r="U10" s="15">
-        <f>S10*(T10*100)</f>
+      <c r="V10" s="15">
+        <f>T10*(U10*100)</f>
         <v>22680</v>
       </c>
-      <c r="V10" s="15">
+      <c r="W10" s="15">
         <f>E10*0.02</f>
         <v>22934.420000000002</v>
       </c>
-      <c r="W10" s="15" t="s">
+      <c r="X10" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="X10" s="16" t="s">
+      <c r="Y10" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="Y10" s="16">
-        <f>(G10-P10)/G10</f>
+      <c r="Z10" s="16">
+        <f>(G10-Q10)/G10</f>
         <v>3.906097418066054E-5</v>
       </c>
-      <c r="Z10" s="16" t="s">
+      <c r="AA10" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="AA10" s="15">
-        <f>S10*1.25</f>
+      <c r="AB10" s="15">
+        <f>T10*1.25</f>
         <v>4.7249999999999996</v>
       </c>
-      <c r="AB10" s="15">
-        <f>(S10*0.25)*(T10*100)</f>
+      <c r="AC10" s="15">
+        <f>(T10*0.25)*(U10*100)</f>
         <v>5670</v>
       </c>
-      <c r="AC10" s="17">
-        <f>S10*0.75</f>
+      <c r="AD10" s="17">
+        <f>T10*0.75</f>
         <v>2.835</v>
       </c>
-      <c r="AD10" s="17">
-        <f>-((S10*0.25)*(T10*100))</f>
+      <c r="AE10" s="17">
+        <f>-((T10*0.25)*(U10*100))</f>
         <v>-5670</v>
       </c>
-      <c r="AE10" s="15">
+      <c r="AF10" s="15">
         <f>G10*0.96</f>
         <v>737.30879999999991</v>
       </c>
-      <c r="AF10" s="15">
+      <c r="AG10" s="15">
         <f>G10*1.04</f>
         <v>798.75120000000004</v>
       </c>
-      <c r="AG10" s="18"/>
-      <c r="AH10" s="7"/>
-      <c r="AI10" s="9"/>
-      <c r="AJ10" s="16">
-        <f>(AI10-G10)/G10</f>
+      <c r="AH10" s="18"/>
+      <c r="AI10" s="7"/>
+      <c r="AJ10" s="9"/>
+      <c r="AK10" s="16">
+        <f>(AJ10-G10)/G10</f>
         <v>-1</v>
       </c>
-      <c r="AK10" s="9"/>
-      <c r="AL10" s="6">
-        <f>AH10-C10</f>
+      <c r="AL10" s="9"/>
+      <c r="AM10" s="6">
+        <f>AI10-C10</f>
         <v>-46295</v>
       </c>
-      <c r="AM10" s="15">
-        <f>((T10*2)*2)*0.65</f>
+      <c r="AN10" s="15">
+        <f>((U10*2)*2)*0.65</f>
         <v>156</v>
       </c>
-      <c r="AN10" s="16">
-        <f>AM10/U10</f>
+      <c r="AO10" s="16">
+        <f>AN10/V10</f>
         <v>6.8783068783068784E-3</v>
       </c>
-      <c r="AO10" s="15">
-        <f>((AK10-S10)*(T10*100))-AM10</f>
+      <c r="AP10" s="15">
+        <f>((AL10-T10)*(U10*100))-AN10</f>
         <v>-22836</v>
       </c>
-      <c r="AP10" s="16">
-        <f>AO10/U10</f>
+      <c r="AQ10" s="16">
+        <f>AP10/V10</f>
         <v>-1.0068783068783069</v>
       </c>
-      <c r="AQ10" s="26">
-        <f>AO10/(E10*0.2)</f>
+      <c r="AR10" s="26">
+        <f>AP10/(E10*0.2)</f>
         <v>-9.9570863357346731E-2</v>
       </c>
-      <c r="AR10" s="16">
-        <f>AO10/E10</f>
+      <c r="AS10" s="16">
+        <f>AP10/E10</f>
         <v>-1.9914172671469346E-2</v>
       </c>
-      <c r="AS10" s="8"/>
+      <c r="AT10" s="8"/>
     </row>
-    <row r="11" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A11" s="5"/>
       <c r="B11" s="6"/>
       <c r="C11" s="7"/>
@@ -5537,45 +5576,46 @@
       <c r="F11" s="10"/>
       <c r="G11" s="9"/>
       <c r="H11" s="7"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="11"/>
-      <c r="K11" s="12"/>
-      <c r="L11" s="13"/>
-      <c r="M11" s="14"/>
+      <c r="I11" s="7"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="11"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="13"/>
       <c r="N11" s="14"/>
-      <c r="O11" s="9"/>
+      <c r="O11" s="14"/>
       <c r="P11" s="9"/>
       <c r="Q11" s="9"/>
       <c r="R11" s="9"/>
       <c r="S11" s="9"/>
-      <c r="T11" s="5"/>
-      <c r="U11" s="15"/>
+      <c r="T11" s="9"/>
+      <c r="U11" s="5"/>
       <c r="V11" s="15"/>
       <c r="W11" s="15"/>
-      <c r="X11" s="16"/>
+      <c r="X11" s="15"/>
       <c r="Y11" s="16"/>
       <c r="Z11" s="16"/>
-      <c r="AA11" s="15"/>
+      <c r="AA11" s="16"/>
       <c r="AB11" s="15"/>
-      <c r="AC11" s="17"/>
+      <c r="AC11" s="15"/>
       <c r="AD11" s="17"/>
-      <c r="AE11" s="15"/>
+      <c r="AE11" s="17"/>
       <c r="AF11" s="15"/>
-      <c r="AG11" s="18"/>
-      <c r="AH11" s="7"/>
-      <c r="AI11" s="9"/>
-      <c r="AJ11" s="15"/>
-      <c r="AK11" s="9"/>
-      <c r="AL11" s="6"/>
-      <c r="AM11" s="15"/>
-      <c r="AN11" s="16"/>
-      <c r="AO11" s="15"/>
-      <c r="AP11" s="16"/>
-      <c r="AQ11" s="26"/>
-      <c r="AR11" s="16"/>
-      <c r="AS11" s="8"/>
+      <c r="AG11" s="15"/>
+      <c r="AH11" s="18"/>
+      <c r="AI11" s="7"/>
+      <c r="AJ11" s="9"/>
+      <c r="AK11" s="15"/>
+      <c r="AL11" s="9"/>
+      <c r="AM11" s="6"/>
+      <c r="AN11" s="15"/>
+      <c r="AO11" s="16"/>
+      <c r="AP11" s="15"/>
+      <c r="AQ11" s="16"/>
+      <c r="AR11" s="26"/>
+      <c r="AS11" s="16"/>
+      <c r="AT11" s="8"/>
     </row>
-    <row r="12" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A12" s="5"/>
       <c r="B12" s="6"/>
       <c r="C12" s="7"/>
@@ -5584,45 +5624,46 @@
       <c r="F12" s="10"/>
       <c r="G12" s="9"/>
       <c r="H12" s="7"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="11"/>
-      <c r="K12" s="12"/>
-      <c r="L12" s="13"/>
-      <c r="M12" s="14"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="5"/>
+      <c r="K12" s="11"/>
+      <c r="L12" s="12"/>
+      <c r="M12" s="13"/>
       <c r="N12" s="14"/>
-      <c r="O12" s="9"/>
+      <c r="O12" s="14"/>
       <c r="P12" s="9"/>
       <c r="Q12" s="9"/>
       <c r="R12" s="9"/>
       <c r="S12" s="9"/>
-      <c r="T12" s="5"/>
-      <c r="U12" s="15"/>
+      <c r="T12" s="9"/>
+      <c r="U12" s="5"/>
       <c r="V12" s="15"/>
       <c r="W12" s="15"/>
-      <c r="X12" s="16"/>
+      <c r="X12" s="15"/>
       <c r="Y12" s="16"/>
       <c r="Z12" s="16"/>
-      <c r="AA12" s="15"/>
+      <c r="AA12" s="16"/>
       <c r="AB12" s="15"/>
-      <c r="AC12" s="17"/>
+      <c r="AC12" s="15"/>
       <c r="AD12" s="17"/>
-      <c r="AE12" s="15"/>
+      <c r="AE12" s="17"/>
       <c r="AF12" s="15"/>
-      <c r="AG12" s="18"/>
-      <c r="AH12" s="7"/>
-      <c r="AI12" s="9"/>
-      <c r="AJ12" s="15"/>
-      <c r="AK12" s="9"/>
-      <c r="AL12" s="6"/>
-      <c r="AM12" s="15"/>
-      <c r="AN12" s="16"/>
-      <c r="AO12" s="15"/>
-      <c r="AP12" s="16"/>
-      <c r="AQ12" s="26"/>
-      <c r="AR12" s="16"/>
-      <c r="AS12" s="8"/>
+      <c r="AG12" s="15"/>
+      <c r="AH12" s="18"/>
+      <c r="AI12" s="7"/>
+      <c r="AJ12" s="9"/>
+      <c r="AK12" s="15"/>
+      <c r="AL12" s="9"/>
+      <c r="AM12" s="6"/>
+      <c r="AN12" s="15"/>
+      <c r="AO12" s="16"/>
+      <c r="AP12" s="15"/>
+      <c r="AQ12" s="16"/>
+      <c r="AR12" s="26"/>
+      <c r="AS12" s="16"/>
+      <c r="AT12" s="8"/>
     </row>
-    <row r="13" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="13" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A13" s="5"/>
       <c r="B13" s="6"/>
       <c r="C13" s="7"/>
@@ -5631,45 +5672,46 @@
       <c r="F13" s="10"/>
       <c r="G13" s="9"/>
       <c r="H13" s="7"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="11"/>
-      <c r="K13" s="12"/>
-      <c r="L13" s="13"/>
-      <c r="M13" s="14"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="11"/>
+      <c r="L13" s="12"/>
+      <c r="M13" s="13"/>
       <c r="N13" s="14"/>
-      <c r="O13" s="9"/>
+      <c r="O13" s="14"/>
       <c r="P13" s="9"/>
       <c r="Q13" s="9"/>
       <c r="R13" s="9"/>
       <c r="S13" s="9"/>
-      <c r="T13" s="5"/>
-      <c r="U13" s="15"/>
+      <c r="T13" s="9"/>
+      <c r="U13" s="5"/>
       <c r="V13" s="15"/>
       <c r="W13" s="15"/>
-      <c r="X13" s="16"/>
+      <c r="X13" s="15"/>
       <c r="Y13" s="16"/>
       <c r="Z13" s="16"/>
-      <c r="AA13" s="15"/>
+      <c r="AA13" s="16"/>
       <c r="AB13" s="15"/>
-      <c r="AC13" s="17"/>
+      <c r="AC13" s="15"/>
       <c r="AD13" s="17"/>
-      <c r="AE13" s="15"/>
+      <c r="AE13" s="17"/>
       <c r="AF13" s="15"/>
-      <c r="AG13" s="18"/>
-      <c r="AH13" s="7"/>
-      <c r="AI13" s="9"/>
-      <c r="AJ13" s="15"/>
-      <c r="AK13" s="9"/>
-      <c r="AL13" s="6"/>
-      <c r="AM13" s="15"/>
-      <c r="AN13" s="16"/>
-      <c r="AO13" s="15"/>
-      <c r="AP13" s="16"/>
-      <c r="AQ13" s="26"/>
-      <c r="AR13" s="16"/>
-      <c r="AS13" s="8"/>
+      <c r="AG13" s="15"/>
+      <c r="AH13" s="18"/>
+      <c r="AI13" s="7"/>
+      <c r="AJ13" s="9"/>
+      <c r="AK13" s="15"/>
+      <c r="AL13" s="9"/>
+      <c r="AM13" s="6"/>
+      <c r="AN13" s="15"/>
+      <c r="AO13" s="16"/>
+      <c r="AP13" s="15"/>
+      <c r="AQ13" s="16"/>
+      <c r="AR13" s="26"/>
+      <c r="AS13" s="16"/>
+      <c r="AT13" s="8"/>
     </row>
-    <row r="14" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="14" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A14" s="5"/>
       <c r="B14" s="6"/>
       <c r="C14" s="7"/>
@@ -5678,45 +5720,46 @@
       <c r="F14" s="10"/>
       <c r="G14" s="9"/>
       <c r="H14" s="7"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="11"/>
-      <c r="K14" s="12"/>
-      <c r="L14" s="13"/>
-      <c r="M14" s="14"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="12"/>
+      <c r="M14" s="13"/>
       <c r="N14" s="14"/>
-      <c r="O14" s="9"/>
+      <c r="O14" s="14"/>
       <c r="P14" s="9"/>
       <c r="Q14" s="9"/>
       <c r="R14" s="9"/>
       <c r="S14" s="9"/>
-      <c r="T14" s="5"/>
-      <c r="U14" s="15"/>
+      <c r="T14" s="9"/>
+      <c r="U14" s="5"/>
       <c r="V14" s="15"/>
       <c r="W14" s="15"/>
-      <c r="X14" s="16"/>
+      <c r="X14" s="15"/>
       <c r="Y14" s="16"/>
       <c r="Z14" s="16"/>
-      <c r="AA14" s="15"/>
+      <c r="AA14" s="16"/>
       <c r="AB14" s="15"/>
-      <c r="AC14" s="17"/>
+      <c r="AC14" s="15"/>
       <c r="AD14" s="17"/>
-      <c r="AE14" s="15"/>
+      <c r="AE14" s="17"/>
       <c r="AF14" s="15"/>
-      <c r="AG14" s="18"/>
-      <c r="AH14" s="7"/>
-      <c r="AI14" s="9"/>
-      <c r="AJ14" s="15"/>
-      <c r="AK14" s="9"/>
-      <c r="AL14" s="6"/>
-      <c r="AM14" s="15"/>
-      <c r="AN14" s="16"/>
-      <c r="AO14" s="15"/>
-      <c r="AP14" s="16"/>
-      <c r="AQ14" s="26"/>
-      <c r="AR14" s="16"/>
-      <c r="AS14" s="8"/>
+      <c r="AG14" s="15"/>
+      <c r="AH14" s="18"/>
+      <c r="AI14" s="7"/>
+      <c r="AJ14" s="9"/>
+      <c r="AK14" s="15"/>
+      <c r="AL14" s="9"/>
+      <c r="AM14" s="6"/>
+      <c r="AN14" s="15"/>
+      <c r="AO14" s="16"/>
+      <c r="AP14" s="15"/>
+      <c r="AQ14" s="16"/>
+      <c r="AR14" s="26"/>
+      <c r="AS14" s="16"/>
+      <c r="AT14" s="8"/>
     </row>
-    <row r="15" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="15" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A15" s="5"/>
       <c r="B15" s="6"/>
       <c r="C15" s="7"/>
@@ -5725,45 +5768,46 @@
       <c r="F15" s="10"/>
       <c r="G15" s="9"/>
       <c r="H15" s="7"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="11"/>
-      <c r="K15" s="12"/>
-      <c r="L15" s="13"/>
-      <c r="M15" s="14"/>
+      <c r="I15" s="7"/>
+      <c r="J15" s="5"/>
+      <c r="K15" s="11"/>
+      <c r="L15" s="12"/>
+      <c r="M15" s="13"/>
       <c r="N15" s="14"/>
-      <c r="O15" s="9"/>
+      <c r="O15" s="14"/>
       <c r="P15" s="9"/>
       <c r="Q15" s="9"/>
       <c r="R15" s="9"/>
       <c r="S15" s="9"/>
-      <c r="T15" s="5"/>
-      <c r="U15" s="15"/>
+      <c r="T15" s="9"/>
+      <c r="U15" s="5"/>
       <c r="V15" s="15"/>
       <c r="W15" s="15"/>
-      <c r="X15" s="16"/>
+      <c r="X15" s="15"/>
       <c r="Y15" s="16"/>
       <c r="Z15" s="16"/>
-      <c r="AA15" s="15"/>
+      <c r="AA15" s="16"/>
       <c r="AB15" s="15"/>
-      <c r="AC15" s="17"/>
+      <c r="AC15" s="15"/>
       <c r="AD15" s="17"/>
-      <c r="AE15" s="15"/>
+      <c r="AE15" s="17"/>
       <c r="AF15" s="15"/>
-      <c r="AG15" s="18"/>
-      <c r="AH15" s="7"/>
-      <c r="AI15" s="9"/>
-      <c r="AJ15" s="15"/>
-      <c r="AK15" s="9"/>
-      <c r="AL15" s="6"/>
-      <c r="AM15" s="15"/>
-      <c r="AN15" s="16"/>
-      <c r="AO15" s="15"/>
-      <c r="AP15" s="16"/>
-      <c r="AQ15" s="26"/>
-      <c r="AR15" s="16"/>
-      <c r="AS15" s="8"/>
+      <c r="AG15" s="15"/>
+      <c r="AH15" s="18"/>
+      <c r="AI15" s="7"/>
+      <c r="AJ15" s="9"/>
+      <c r="AK15" s="15"/>
+      <c r="AL15" s="9"/>
+      <c r="AM15" s="6"/>
+      <c r="AN15" s="15"/>
+      <c r="AO15" s="16"/>
+      <c r="AP15" s="15"/>
+      <c r="AQ15" s="16"/>
+      <c r="AR15" s="26"/>
+      <c r="AS15" s="16"/>
+      <c r="AT15" s="8"/>
     </row>
-    <row r="16" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="16" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A16" s="5"/>
       <c r="B16" s="6"/>
       <c r="C16" s="7"/>
@@ -5772,45 +5816,46 @@
       <c r="F16" s="10"/>
       <c r="G16" s="9"/>
       <c r="H16" s="7"/>
-      <c r="I16" s="5"/>
-      <c r="J16" s="11"/>
-      <c r="K16" s="12"/>
-      <c r="L16" s="13"/>
-      <c r="M16" s="14"/>
+      <c r="I16" s="7"/>
+      <c r="J16" s="5"/>
+      <c r="K16" s="11"/>
+      <c r="L16" s="12"/>
+      <c r="M16" s="13"/>
       <c r="N16" s="14"/>
-      <c r="O16" s="9"/>
+      <c r="O16" s="14"/>
       <c r="P16" s="9"/>
       <c r="Q16" s="9"/>
       <c r="R16" s="9"/>
       <c r="S16" s="9"/>
-      <c r="T16" s="5"/>
-      <c r="U16" s="15"/>
+      <c r="T16" s="9"/>
+      <c r="U16" s="5"/>
       <c r="V16" s="15"/>
       <c r="W16" s="15"/>
-      <c r="X16" s="16"/>
+      <c r="X16" s="15"/>
       <c r="Y16" s="16"/>
       <c r="Z16" s="16"/>
-      <c r="AA16" s="15"/>
+      <c r="AA16" s="16"/>
       <c r="AB16" s="15"/>
-      <c r="AC16" s="17"/>
+      <c r="AC16" s="15"/>
       <c r="AD16" s="17"/>
-      <c r="AE16" s="15"/>
+      <c r="AE16" s="17"/>
       <c r="AF16" s="15"/>
-      <c r="AG16" s="18"/>
-      <c r="AH16" s="7"/>
-      <c r="AI16" s="9"/>
-      <c r="AJ16" s="15"/>
-      <c r="AK16" s="9"/>
-      <c r="AL16" s="6"/>
-      <c r="AM16" s="15"/>
-      <c r="AN16" s="16"/>
-      <c r="AO16" s="15"/>
-      <c r="AP16" s="16"/>
-      <c r="AQ16" s="26"/>
-      <c r="AR16" s="16"/>
-      <c r="AS16" s="8"/>
+      <c r="AG16" s="15"/>
+      <c r="AH16" s="18"/>
+      <c r="AI16" s="7"/>
+      <c r="AJ16" s="9"/>
+      <c r="AK16" s="15"/>
+      <c r="AL16" s="9"/>
+      <c r="AM16" s="6"/>
+      <c r="AN16" s="15"/>
+      <c r="AO16" s="16"/>
+      <c r="AP16" s="15"/>
+      <c r="AQ16" s="16"/>
+      <c r="AR16" s="26"/>
+      <c r="AS16" s="16"/>
+      <c r="AT16" s="8"/>
     </row>
-    <row r="17" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="17" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A17" s="5"/>
       <c r="B17" s="6"/>
       <c r="C17" s="7"/>
@@ -5819,45 +5864,46 @@
       <c r="F17" s="10"/>
       <c r="G17" s="9"/>
       <c r="H17" s="7"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="11"/>
-      <c r="K17" s="12"/>
-      <c r="L17" s="13"/>
-      <c r="M17" s="14"/>
+      <c r="I17" s="7"/>
+      <c r="J17" s="5"/>
+      <c r="K17" s="11"/>
+      <c r="L17" s="12"/>
+      <c r="M17" s="13"/>
       <c r="N17" s="14"/>
-      <c r="O17" s="9"/>
+      <c r="O17" s="14"/>
       <c r="P17" s="9"/>
       <c r="Q17" s="9"/>
       <c r="R17" s="9"/>
       <c r="S17" s="9"/>
-      <c r="T17" s="5"/>
-      <c r="U17" s="15"/>
+      <c r="T17" s="9"/>
+      <c r="U17" s="5"/>
       <c r="V17" s="15"/>
       <c r="W17" s="15"/>
-      <c r="X17" s="16"/>
+      <c r="X17" s="15"/>
       <c r="Y17" s="16"/>
       <c r="Z17" s="16"/>
-      <c r="AA17" s="15"/>
+      <c r="AA17" s="16"/>
       <c r="AB17" s="15"/>
-      <c r="AC17" s="17"/>
+      <c r="AC17" s="15"/>
       <c r="AD17" s="17"/>
-      <c r="AE17" s="15"/>
+      <c r="AE17" s="17"/>
       <c r="AF17" s="15"/>
-      <c r="AG17" s="18"/>
-      <c r="AH17" s="7"/>
-      <c r="AI17" s="9"/>
-      <c r="AJ17" s="15"/>
-      <c r="AK17" s="9"/>
-      <c r="AL17" s="6"/>
-      <c r="AM17" s="15"/>
-      <c r="AN17" s="16"/>
-      <c r="AO17" s="15"/>
-      <c r="AP17" s="16"/>
-      <c r="AQ17" s="26"/>
-      <c r="AR17" s="16"/>
-      <c r="AS17" s="8"/>
+      <c r="AG17" s="15"/>
+      <c r="AH17" s="18"/>
+      <c r="AI17" s="7"/>
+      <c r="AJ17" s="9"/>
+      <c r="AK17" s="15"/>
+      <c r="AL17" s="9"/>
+      <c r="AM17" s="6"/>
+      <c r="AN17" s="15"/>
+      <c r="AO17" s="16"/>
+      <c r="AP17" s="15"/>
+      <c r="AQ17" s="16"/>
+      <c r="AR17" s="26"/>
+      <c r="AS17" s="16"/>
+      <c r="AT17" s="8"/>
     </row>
-    <row r="18" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="18" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A18" s="5"/>
       <c r="B18" s="6"/>
       <c r="C18" s="7"/>
@@ -5866,45 +5912,46 @@
       <c r="F18" s="10"/>
       <c r="G18" s="9"/>
       <c r="H18" s="7"/>
-      <c r="I18" s="5"/>
-      <c r="J18" s="11"/>
-      <c r="K18" s="12"/>
-      <c r="L18" s="13"/>
-      <c r="M18" s="14"/>
+      <c r="I18" s="7"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="11"/>
+      <c r="L18" s="12"/>
+      <c r="M18" s="13"/>
       <c r="N18" s="14"/>
-      <c r="O18" s="9"/>
+      <c r="O18" s="14"/>
       <c r="P18" s="9"/>
       <c r="Q18" s="9"/>
       <c r="R18" s="9"/>
       <c r="S18" s="9"/>
-      <c r="T18" s="5"/>
-      <c r="U18" s="15"/>
+      <c r="T18" s="9"/>
+      <c r="U18" s="5"/>
       <c r="V18" s="15"/>
       <c r="W18" s="15"/>
-      <c r="X18" s="16"/>
+      <c r="X18" s="15"/>
       <c r="Y18" s="16"/>
       <c r="Z18" s="16"/>
-      <c r="AA18" s="15"/>
+      <c r="AA18" s="16"/>
       <c r="AB18" s="15"/>
-      <c r="AC18" s="17"/>
+      <c r="AC18" s="15"/>
       <c r="AD18" s="17"/>
-      <c r="AE18" s="15"/>
+      <c r="AE18" s="17"/>
       <c r="AF18" s="15"/>
-      <c r="AG18" s="18"/>
-      <c r="AH18" s="7"/>
-      <c r="AI18" s="9"/>
-      <c r="AJ18" s="15"/>
-      <c r="AK18" s="9"/>
-      <c r="AL18" s="6"/>
-      <c r="AM18" s="15"/>
-      <c r="AN18" s="16"/>
-      <c r="AO18" s="15"/>
-      <c r="AP18" s="16"/>
-      <c r="AQ18" s="26"/>
-      <c r="AR18" s="16"/>
-      <c r="AS18" s="8"/>
+      <c r="AG18" s="15"/>
+      <c r="AH18" s="18"/>
+      <c r="AI18" s="7"/>
+      <c r="AJ18" s="9"/>
+      <c r="AK18" s="15"/>
+      <c r="AL18" s="9"/>
+      <c r="AM18" s="6"/>
+      <c r="AN18" s="15"/>
+      <c r="AO18" s="16"/>
+      <c r="AP18" s="15"/>
+      <c r="AQ18" s="16"/>
+      <c r="AR18" s="26"/>
+      <c r="AS18" s="16"/>
+      <c r="AT18" s="8"/>
     </row>
-    <row r="19" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="19" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A19" s="5"/>
       <c r="B19" s="6"/>
       <c r="C19" s="7"/>
@@ -5913,45 +5960,46 @@
       <c r="F19" s="10"/>
       <c r="G19" s="9"/>
       <c r="H19" s="7"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="11"/>
-      <c r="K19" s="12"/>
-      <c r="L19" s="13"/>
-      <c r="M19" s="14"/>
+      <c r="I19" s="7"/>
+      <c r="J19" s="5"/>
+      <c r="K19" s="11"/>
+      <c r="L19" s="12"/>
+      <c r="M19" s="13"/>
       <c r="N19" s="14"/>
-      <c r="O19" s="9"/>
+      <c r="O19" s="14"/>
       <c r="P19" s="9"/>
       <c r="Q19" s="9"/>
       <c r="R19" s="9"/>
       <c r="S19" s="9"/>
-      <c r="T19" s="5"/>
-      <c r="U19" s="15"/>
+      <c r="T19" s="9"/>
+      <c r="U19" s="5"/>
       <c r="V19" s="15"/>
       <c r="W19" s="15"/>
-      <c r="X19" s="16"/>
+      <c r="X19" s="15"/>
       <c r="Y19" s="16"/>
       <c r="Z19" s="16"/>
-      <c r="AA19" s="15"/>
+      <c r="AA19" s="16"/>
       <c r="AB19" s="15"/>
-      <c r="AC19" s="17"/>
+      <c r="AC19" s="15"/>
       <c r="AD19" s="17"/>
-      <c r="AE19" s="15"/>
+      <c r="AE19" s="17"/>
       <c r="AF19" s="15"/>
-      <c r="AG19" s="18"/>
-      <c r="AH19" s="7"/>
-      <c r="AI19" s="9"/>
-      <c r="AJ19" s="15"/>
-      <c r="AK19" s="9"/>
-      <c r="AL19" s="6"/>
-      <c r="AM19" s="15"/>
-      <c r="AN19" s="16"/>
-      <c r="AO19" s="15"/>
-      <c r="AP19" s="16"/>
-      <c r="AQ19" s="26"/>
-      <c r="AR19" s="16"/>
-      <c r="AS19" s="8"/>
+      <c r="AG19" s="15"/>
+      <c r="AH19" s="18"/>
+      <c r="AI19" s="7"/>
+      <c r="AJ19" s="9"/>
+      <c r="AK19" s="15"/>
+      <c r="AL19" s="9"/>
+      <c r="AM19" s="6"/>
+      <c r="AN19" s="15"/>
+      <c r="AO19" s="16"/>
+      <c r="AP19" s="15"/>
+      <c r="AQ19" s="16"/>
+      <c r="AR19" s="26"/>
+      <c r="AS19" s="16"/>
+      <c r="AT19" s="8"/>
     </row>
-    <row r="20" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="20" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A20" s="5"/>
       <c r="B20" s="6"/>
       <c r="C20" s="7"/>
@@ -5960,45 +6008,46 @@
       <c r="F20" s="10"/>
       <c r="G20" s="9"/>
       <c r="H20" s="7"/>
-      <c r="I20" s="5"/>
-      <c r="J20" s="11"/>
-      <c r="K20" s="12"/>
-      <c r="L20" s="13"/>
-      <c r="M20" s="14"/>
+      <c r="I20" s="7"/>
+      <c r="J20" s="5"/>
+      <c r="K20" s="11"/>
+      <c r="L20" s="12"/>
+      <c r="M20" s="13"/>
       <c r="N20" s="14"/>
-      <c r="O20" s="9"/>
+      <c r="O20" s="14"/>
       <c r="P20" s="9"/>
       <c r="Q20" s="9"/>
       <c r="R20" s="9"/>
       <c r="S20" s="9"/>
-      <c r="T20" s="5"/>
-      <c r="U20" s="15"/>
+      <c r="T20" s="9"/>
+      <c r="U20" s="5"/>
       <c r="V20" s="15"/>
       <c r="W20" s="15"/>
-      <c r="X20" s="16"/>
+      <c r="X20" s="15"/>
       <c r="Y20" s="16"/>
       <c r="Z20" s="16"/>
-      <c r="AA20" s="15"/>
+      <c r="AA20" s="16"/>
       <c r="AB20" s="15"/>
-      <c r="AC20" s="17"/>
+      <c r="AC20" s="15"/>
       <c r="AD20" s="17"/>
-      <c r="AE20" s="15"/>
+      <c r="AE20" s="17"/>
       <c r="AF20" s="15"/>
-      <c r="AG20" s="18"/>
-      <c r="AH20" s="7"/>
-      <c r="AI20" s="9"/>
-      <c r="AJ20" s="15"/>
-      <c r="AK20" s="9"/>
-      <c r="AL20" s="6"/>
-      <c r="AM20" s="15"/>
-      <c r="AN20" s="16"/>
-      <c r="AO20" s="15"/>
-      <c r="AP20" s="16"/>
-      <c r="AQ20" s="26"/>
-      <c r="AR20" s="16"/>
-      <c r="AS20" s="8"/>
+      <c r="AG20" s="15"/>
+      <c r="AH20" s="18"/>
+      <c r="AI20" s="7"/>
+      <c r="AJ20" s="9"/>
+      <c r="AK20" s="15"/>
+      <c r="AL20" s="9"/>
+      <c r="AM20" s="6"/>
+      <c r="AN20" s="15"/>
+      <c r="AO20" s="16"/>
+      <c r="AP20" s="15"/>
+      <c r="AQ20" s="16"/>
+      <c r="AR20" s="26"/>
+      <c r="AS20" s="16"/>
+      <c r="AT20" s="8"/>
     </row>
-    <row r="21" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="21" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A21" s="5"/>
       <c r="B21" s="6"/>
       <c r="C21" s="7"/>
@@ -6007,45 +6056,46 @@
       <c r="F21" s="10"/>
       <c r="G21" s="9"/>
       <c r="H21" s="7"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="11"/>
-      <c r="K21" s="12"/>
-      <c r="L21" s="13"/>
-      <c r="M21" s="14"/>
+      <c r="I21" s="7"/>
+      <c r="J21" s="5"/>
+      <c r="K21" s="11"/>
+      <c r="L21" s="12"/>
+      <c r="M21" s="13"/>
       <c r="N21" s="14"/>
-      <c r="O21" s="9"/>
+      <c r="O21" s="14"/>
       <c r="P21" s="9"/>
       <c r="Q21" s="9"/>
       <c r="R21" s="9"/>
       <c r="S21" s="9"/>
-      <c r="T21" s="5"/>
-      <c r="U21" s="15"/>
+      <c r="T21" s="9"/>
+      <c r="U21" s="5"/>
       <c r="V21" s="15"/>
       <c r="W21" s="15"/>
-      <c r="X21" s="16"/>
+      <c r="X21" s="15"/>
       <c r="Y21" s="16"/>
       <c r="Z21" s="16"/>
-      <c r="AA21" s="15"/>
+      <c r="AA21" s="16"/>
       <c r="AB21" s="15"/>
-      <c r="AC21" s="17"/>
+      <c r="AC21" s="15"/>
       <c r="AD21" s="17"/>
-      <c r="AE21" s="15"/>
+      <c r="AE21" s="17"/>
       <c r="AF21" s="15"/>
-      <c r="AG21" s="18"/>
-      <c r="AH21" s="7"/>
-      <c r="AI21" s="9"/>
-      <c r="AJ21" s="15"/>
-      <c r="AK21" s="9"/>
-      <c r="AL21" s="6"/>
-      <c r="AM21" s="15"/>
-      <c r="AN21" s="16"/>
-      <c r="AO21" s="15"/>
-      <c r="AP21" s="16"/>
-      <c r="AQ21" s="26"/>
-      <c r="AR21" s="16"/>
-      <c r="AS21" s="8"/>
+      <c r="AG21" s="15"/>
+      <c r="AH21" s="18"/>
+      <c r="AI21" s="7"/>
+      <c r="AJ21" s="9"/>
+      <c r="AK21" s="15"/>
+      <c r="AL21" s="9"/>
+      <c r="AM21" s="6"/>
+      <c r="AN21" s="15"/>
+      <c r="AO21" s="16"/>
+      <c r="AP21" s="15"/>
+      <c r="AQ21" s="16"/>
+      <c r="AR21" s="26"/>
+      <c r="AS21" s="16"/>
+      <c r="AT21" s="8"/>
     </row>
-    <row r="22" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="22" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A22" s="5"/>
       <c r="B22" s="6"/>
       <c r="C22" s="7"/>
@@ -6054,45 +6104,46 @@
       <c r="F22" s="10"/>
       <c r="G22" s="9"/>
       <c r="H22" s="7"/>
-      <c r="I22" s="5"/>
-      <c r="J22" s="11"/>
-      <c r="K22" s="12"/>
-      <c r="L22" s="13"/>
-      <c r="M22" s="14"/>
+      <c r="I22" s="7"/>
+      <c r="J22" s="5"/>
+      <c r="K22" s="11"/>
+      <c r="L22" s="12"/>
+      <c r="M22" s="13"/>
       <c r="N22" s="14"/>
-      <c r="O22" s="9"/>
+      <c r="O22" s="14"/>
       <c r="P22" s="9"/>
       <c r="Q22" s="9"/>
       <c r="R22" s="9"/>
       <c r="S22" s="9"/>
-      <c r="T22" s="5"/>
-      <c r="U22" s="15"/>
+      <c r="T22" s="9"/>
+      <c r="U22" s="5"/>
       <c r="V22" s="15"/>
       <c r="W22" s="15"/>
-      <c r="X22" s="16"/>
+      <c r="X22" s="15"/>
       <c r="Y22" s="16"/>
       <c r="Z22" s="16"/>
-      <c r="AA22" s="15"/>
+      <c r="AA22" s="16"/>
       <c r="AB22" s="15"/>
-      <c r="AC22" s="17"/>
+      <c r="AC22" s="15"/>
       <c r="AD22" s="17"/>
-      <c r="AE22" s="15"/>
+      <c r="AE22" s="17"/>
       <c r="AF22" s="15"/>
-      <c r="AG22" s="18"/>
-      <c r="AH22" s="7"/>
-      <c r="AI22" s="9"/>
-      <c r="AJ22" s="15"/>
-      <c r="AK22" s="9"/>
-      <c r="AL22" s="6"/>
-      <c r="AM22" s="15"/>
-      <c r="AN22" s="16"/>
-      <c r="AO22" s="15"/>
-      <c r="AP22" s="16"/>
-      <c r="AQ22" s="26"/>
-      <c r="AR22" s="16"/>
-      <c r="AS22" s="8"/>
+      <c r="AG22" s="15"/>
+      <c r="AH22" s="18"/>
+      <c r="AI22" s="7"/>
+      <c r="AJ22" s="9"/>
+      <c r="AK22" s="15"/>
+      <c r="AL22" s="9"/>
+      <c r="AM22" s="6"/>
+      <c r="AN22" s="15"/>
+      <c r="AO22" s="16"/>
+      <c r="AP22" s="15"/>
+      <c r="AQ22" s="16"/>
+      <c r="AR22" s="26"/>
+      <c r="AS22" s="16"/>
+      <c r="AT22" s="8"/>
     </row>
-    <row r="23" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="23" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A23" s="5"/>
       <c r="B23" s="6"/>
       <c r="C23" s="7"/>
@@ -6101,45 +6152,46 @@
       <c r="F23" s="10"/>
       <c r="G23" s="9"/>
       <c r="H23" s="7"/>
-      <c r="I23" s="5"/>
-      <c r="J23" s="11"/>
-      <c r="K23" s="12"/>
-      <c r="L23" s="13"/>
-      <c r="M23" s="14"/>
+      <c r="I23" s="7"/>
+      <c r="J23" s="5"/>
+      <c r="K23" s="11"/>
+      <c r="L23" s="12"/>
+      <c r="M23" s="13"/>
       <c r="N23" s="14"/>
-      <c r="O23" s="9"/>
+      <c r="O23" s="14"/>
       <c r="P23" s="9"/>
       <c r="Q23" s="9"/>
       <c r="R23" s="9"/>
       <c r="S23" s="9"/>
-      <c r="T23" s="5"/>
-      <c r="U23" s="15"/>
+      <c r="T23" s="9"/>
+      <c r="U23" s="5"/>
       <c r="V23" s="15"/>
       <c r="W23" s="15"/>
-      <c r="X23" s="16"/>
+      <c r="X23" s="15"/>
       <c r="Y23" s="16"/>
       <c r="Z23" s="16"/>
-      <c r="AA23" s="15"/>
+      <c r="AA23" s="16"/>
       <c r="AB23" s="15"/>
-      <c r="AC23" s="17"/>
+      <c r="AC23" s="15"/>
       <c r="AD23" s="17"/>
-      <c r="AE23" s="15"/>
+      <c r="AE23" s="17"/>
       <c r="AF23" s="15"/>
-      <c r="AG23" s="18"/>
-      <c r="AH23" s="7"/>
-      <c r="AI23" s="9"/>
-      <c r="AJ23" s="15"/>
-      <c r="AK23" s="9"/>
-      <c r="AL23" s="6"/>
-      <c r="AM23" s="15"/>
-      <c r="AN23" s="16"/>
-      <c r="AO23" s="15"/>
-      <c r="AP23" s="16"/>
-      <c r="AQ23" s="26"/>
-      <c r="AR23" s="16"/>
-      <c r="AS23" s="8"/>
+      <c r="AG23" s="15"/>
+      <c r="AH23" s="18"/>
+      <c r="AI23" s="7"/>
+      <c r="AJ23" s="9"/>
+      <c r="AK23" s="15"/>
+      <c r="AL23" s="9"/>
+      <c r="AM23" s="6"/>
+      <c r="AN23" s="15"/>
+      <c r="AO23" s="16"/>
+      <c r="AP23" s="15"/>
+      <c r="AQ23" s="16"/>
+      <c r="AR23" s="26"/>
+      <c r="AS23" s="16"/>
+      <c r="AT23" s="8"/>
     </row>
-    <row r="24" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="24" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A24" s="5"/>
       <c r="B24" s="6"/>
       <c r="C24" s="7"/>
@@ -6148,45 +6200,46 @@
       <c r="F24" s="10"/>
       <c r="G24" s="9"/>
       <c r="H24" s="7"/>
-      <c r="I24" s="5"/>
-      <c r="J24" s="11"/>
-      <c r="K24" s="12"/>
-      <c r="L24" s="13"/>
-      <c r="M24" s="14"/>
+      <c r="I24" s="7"/>
+      <c r="J24" s="5"/>
+      <c r="K24" s="11"/>
+      <c r="L24" s="12"/>
+      <c r="M24" s="13"/>
       <c r="N24" s="14"/>
-      <c r="O24" s="9"/>
+      <c r="O24" s="14"/>
       <c r="P24" s="9"/>
       <c r="Q24" s="9"/>
       <c r="R24" s="9"/>
       <c r="S24" s="9"/>
-      <c r="T24" s="5"/>
-      <c r="U24" s="15"/>
+      <c r="T24" s="9"/>
+      <c r="U24" s="5"/>
       <c r="V24" s="15"/>
       <c r="W24" s="15"/>
-      <c r="X24" s="16"/>
+      <c r="X24" s="15"/>
       <c r="Y24" s="16"/>
       <c r="Z24" s="16"/>
-      <c r="AA24" s="15"/>
+      <c r="AA24" s="16"/>
       <c r="AB24" s="15"/>
-      <c r="AC24" s="17"/>
+      <c r="AC24" s="15"/>
       <c r="AD24" s="17"/>
-      <c r="AE24" s="15"/>
+      <c r="AE24" s="17"/>
       <c r="AF24" s="15"/>
-      <c r="AG24" s="18"/>
-      <c r="AH24" s="7"/>
-      <c r="AI24" s="9"/>
-      <c r="AJ24" s="15"/>
-      <c r="AK24" s="9"/>
-      <c r="AL24" s="6"/>
-      <c r="AM24" s="15"/>
-      <c r="AN24" s="16"/>
-      <c r="AO24" s="15"/>
-      <c r="AP24" s="16"/>
-      <c r="AQ24" s="26"/>
-      <c r="AR24" s="16"/>
-      <c r="AS24" s="8"/>
+      <c r="AG24" s="15"/>
+      <c r="AH24" s="18"/>
+      <c r="AI24" s="7"/>
+      <c r="AJ24" s="9"/>
+      <c r="AK24" s="15"/>
+      <c r="AL24" s="9"/>
+      <c r="AM24" s="6"/>
+      <c r="AN24" s="15"/>
+      <c r="AO24" s="16"/>
+      <c r="AP24" s="15"/>
+      <c r="AQ24" s="16"/>
+      <c r="AR24" s="26"/>
+      <c r="AS24" s="16"/>
+      <c r="AT24" s="8"/>
     </row>
-    <row r="25" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="25" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A25" s="5"/>
       <c r="B25" s="6"/>
       <c r="C25" s="7"/>
@@ -6195,45 +6248,46 @@
       <c r="F25" s="10"/>
       <c r="G25" s="9"/>
       <c r="H25" s="7"/>
-      <c r="I25" s="5"/>
-      <c r="J25" s="11"/>
-      <c r="K25" s="12"/>
-      <c r="L25" s="13"/>
-      <c r="M25" s="14"/>
+      <c r="I25" s="7"/>
+      <c r="J25" s="5"/>
+      <c r="K25" s="11"/>
+      <c r="L25" s="12"/>
+      <c r="M25" s="13"/>
       <c r="N25" s="14"/>
-      <c r="O25" s="9"/>
+      <c r="O25" s="14"/>
       <c r="P25" s="9"/>
       <c r="Q25" s="9"/>
       <c r="R25" s="9"/>
       <c r="S25" s="9"/>
-      <c r="T25" s="5"/>
-      <c r="U25" s="15"/>
+      <c r="T25" s="9"/>
+      <c r="U25" s="5"/>
       <c r="V25" s="15"/>
       <c r="W25" s="15"/>
-      <c r="X25" s="16"/>
+      <c r="X25" s="15"/>
       <c r="Y25" s="16"/>
       <c r="Z25" s="16"/>
-      <c r="AA25" s="15"/>
+      <c r="AA25" s="16"/>
       <c r="AB25" s="15"/>
-      <c r="AC25" s="17"/>
+      <c r="AC25" s="15"/>
       <c r="AD25" s="17"/>
-      <c r="AE25" s="15"/>
+      <c r="AE25" s="17"/>
       <c r="AF25" s="15"/>
-      <c r="AG25" s="18"/>
-      <c r="AH25" s="7"/>
-      <c r="AI25" s="9"/>
-      <c r="AJ25" s="15"/>
-      <c r="AK25" s="9"/>
-      <c r="AL25" s="6"/>
-      <c r="AM25" s="15"/>
-      <c r="AN25" s="16"/>
-      <c r="AO25" s="15"/>
-      <c r="AP25" s="16"/>
-      <c r="AQ25" s="26"/>
-      <c r="AR25" s="16"/>
-      <c r="AS25" s="8"/>
+      <c r="AG25" s="15"/>
+      <c r="AH25" s="18"/>
+      <c r="AI25" s="7"/>
+      <c r="AJ25" s="9"/>
+      <c r="AK25" s="15"/>
+      <c r="AL25" s="9"/>
+      <c r="AM25" s="6"/>
+      <c r="AN25" s="15"/>
+      <c r="AO25" s="16"/>
+      <c r="AP25" s="15"/>
+      <c r="AQ25" s="16"/>
+      <c r="AR25" s="26"/>
+      <c r="AS25" s="16"/>
+      <c r="AT25" s="8"/>
     </row>
-    <row r="26" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="26" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A26" s="5"/>
       <c r="B26" s="6"/>
       <c r="C26" s="7"/>
@@ -6242,45 +6296,46 @@
       <c r="F26" s="10"/>
       <c r="G26" s="9"/>
       <c r="H26" s="7"/>
-      <c r="I26" s="5"/>
-      <c r="J26" s="11"/>
-      <c r="K26" s="12"/>
-      <c r="L26" s="13"/>
-      <c r="M26" s="14"/>
+      <c r="I26" s="7"/>
+      <c r="J26" s="5"/>
+      <c r="K26" s="11"/>
+      <c r="L26" s="12"/>
+      <c r="M26" s="13"/>
       <c r="N26" s="14"/>
-      <c r="O26" s="9"/>
+      <c r="O26" s="14"/>
       <c r="P26" s="9"/>
       <c r="Q26" s="9"/>
       <c r="R26" s="9"/>
       <c r="S26" s="9"/>
-      <c r="T26" s="5"/>
-      <c r="U26" s="15"/>
+      <c r="T26" s="9"/>
+      <c r="U26" s="5"/>
       <c r="V26" s="15"/>
       <c r="W26" s="15"/>
-      <c r="X26" s="16"/>
+      <c r="X26" s="15"/>
       <c r="Y26" s="16"/>
       <c r="Z26" s="16"/>
-      <c r="AA26" s="15"/>
+      <c r="AA26" s="16"/>
       <c r="AB26" s="15"/>
-      <c r="AC26" s="17"/>
+      <c r="AC26" s="15"/>
       <c r="AD26" s="17"/>
-      <c r="AE26" s="15"/>
+      <c r="AE26" s="17"/>
       <c r="AF26" s="15"/>
-      <c r="AG26" s="18"/>
-      <c r="AH26" s="7"/>
-      <c r="AI26" s="9"/>
-      <c r="AJ26" s="15"/>
-      <c r="AK26" s="9"/>
-      <c r="AL26" s="6"/>
-      <c r="AM26" s="15"/>
-      <c r="AN26" s="16"/>
-      <c r="AO26" s="15"/>
-      <c r="AP26" s="16"/>
-      <c r="AQ26" s="26"/>
-      <c r="AR26" s="16"/>
-      <c r="AS26" s="8"/>
+      <c r="AG26" s="15"/>
+      <c r="AH26" s="18"/>
+      <c r="AI26" s="7"/>
+      <c r="AJ26" s="9"/>
+      <c r="AK26" s="15"/>
+      <c r="AL26" s="9"/>
+      <c r="AM26" s="6"/>
+      <c r="AN26" s="15"/>
+      <c r="AO26" s="16"/>
+      <c r="AP26" s="15"/>
+      <c r="AQ26" s="16"/>
+      <c r="AR26" s="26"/>
+      <c r="AS26" s="16"/>
+      <c r="AT26" s="8"/>
     </row>
-    <row r="27" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="27" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A27" s="5"/>
       <c r="B27" s="6"/>
       <c r="C27" s="7"/>
@@ -6289,45 +6344,46 @@
       <c r="F27" s="10"/>
       <c r="G27" s="9"/>
       <c r="H27" s="7"/>
-      <c r="I27" s="5"/>
-      <c r="J27" s="11"/>
-      <c r="K27" s="12"/>
-      <c r="L27" s="13"/>
-      <c r="M27" s="14"/>
+      <c r="I27" s="7"/>
+      <c r="J27" s="5"/>
+      <c r="K27" s="11"/>
+      <c r="L27" s="12"/>
+      <c r="M27" s="13"/>
       <c r="N27" s="14"/>
-      <c r="O27" s="9"/>
+      <c r="O27" s="14"/>
       <c r="P27" s="9"/>
       <c r="Q27" s="9"/>
       <c r="R27" s="9"/>
       <c r="S27" s="9"/>
-      <c r="T27" s="5"/>
-      <c r="U27" s="15"/>
+      <c r="T27" s="9"/>
+      <c r="U27" s="5"/>
       <c r="V27" s="15"/>
       <c r="W27" s="15"/>
-      <c r="X27" s="16"/>
+      <c r="X27" s="15"/>
       <c r="Y27" s="16"/>
       <c r="Z27" s="16"/>
-      <c r="AA27" s="15"/>
+      <c r="AA27" s="16"/>
       <c r="AB27" s="15"/>
-      <c r="AC27" s="17"/>
+      <c r="AC27" s="15"/>
       <c r="AD27" s="17"/>
-      <c r="AE27" s="15"/>
+      <c r="AE27" s="17"/>
       <c r="AF27" s="15"/>
-      <c r="AG27" s="18"/>
-      <c r="AH27" s="7"/>
-      <c r="AI27" s="9"/>
-      <c r="AJ27" s="15"/>
-      <c r="AK27" s="9"/>
-      <c r="AL27" s="6"/>
-      <c r="AM27" s="15"/>
-      <c r="AN27" s="16"/>
-      <c r="AO27" s="15"/>
-      <c r="AP27" s="16"/>
-      <c r="AQ27" s="26"/>
-      <c r="AR27" s="16"/>
-      <c r="AS27" s="8"/>
+      <c r="AG27" s="15"/>
+      <c r="AH27" s="18"/>
+      <c r="AI27" s="7"/>
+      <c r="AJ27" s="9"/>
+      <c r="AK27" s="15"/>
+      <c r="AL27" s="9"/>
+      <c r="AM27" s="6"/>
+      <c r="AN27" s="15"/>
+      <c r="AO27" s="16"/>
+      <c r="AP27" s="15"/>
+      <c r="AQ27" s="16"/>
+      <c r="AR27" s="26"/>
+      <c r="AS27" s="16"/>
+      <c r="AT27" s="8"/>
     </row>
-    <row r="28" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="28" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A28" s="5"/>
       <c r="B28" s="6"/>
       <c r="C28" s="7"/>
@@ -6336,45 +6392,46 @@
       <c r="F28" s="10"/>
       <c r="G28" s="9"/>
       <c r="H28" s="7"/>
-      <c r="I28" s="5"/>
-      <c r="J28" s="11"/>
-      <c r="K28" s="12"/>
-      <c r="L28" s="13"/>
-      <c r="M28" s="14"/>
+      <c r="I28" s="7"/>
+      <c r="J28" s="5"/>
+      <c r="K28" s="11"/>
+      <c r="L28" s="12"/>
+      <c r="M28" s="13"/>
       <c r="N28" s="14"/>
-      <c r="O28" s="9"/>
+      <c r="O28" s="14"/>
       <c r="P28" s="9"/>
       <c r="Q28" s="9"/>
       <c r="R28" s="9"/>
       <c r="S28" s="9"/>
-      <c r="T28" s="5"/>
-      <c r="U28" s="15"/>
+      <c r="T28" s="9"/>
+      <c r="U28" s="5"/>
       <c r="V28" s="15"/>
       <c r="W28" s="15"/>
-      <c r="X28" s="16"/>
+      <c r="X28" s="15"/>
       <c r="Y28" s="16"/>
       <c r="Z28" s="16"/>
-      <c r="AA28" s="15"/>
+      <c r="AA28" s="16"/>
       <c r="AB28" s="15"/>
-      <c r="AC28" s="17"/>
+      <c r="AC28" s="15"/>
       <c r="AD28" s="17"/>
-      <c r="AE28" s="15"/>
+      <c r="AE28" s="17"/>
       <c r="AF28" s="15"/>
-      <c r="AG28" s="18"/>
-      <c r="AH28" s="7"/>
-      <c r="AI28" s="9"/>
-      <c r="AJ28" s="15"/>
-      <c r="AK28" s="9"/>
-      <c r="AL28" s="6"/>
-      <c r="AM28" s="15"/>
-      <c r="AN28" s="16"/>
-      <c r="AO28" s="15"/>
-      <c r="AP28" s="16"/>
-      <c r="AQ28" s="26"/>
-      <c r="AR28" s="16"/>
-      <c r="AS28" s="8"/>
+      <c r="AG28" s="15"/>
+      <c r="AH28" s="18"/>
+      <c r="AI28" s="7"/>
+      <c r="AJ28" s="9"/>
+      <c r="AK28" s="15"/>
+      <c r="AL28" s="9"/>
+      <c r="AM28" s="6"/>
+      <c r="AN28" s="15"/>
+      <c r="AO28" s="16"/>
+      <c r="AP28" s="15"/>
+      <c r="AQ28" s="16"/>
+      <c r="AR28" s="26"/>
+      <c r="AS28" s="16"/>
+      <c r="AT28" s="8"/>
     </row>
-    <row r="29" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="29" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A29" s="5"/>
       <c r="B29" s="6"/>
       <c r="C29" s="7"/>
@@ -6383,45 +6440,46 @@
       <c r="F29" s="10"/>
       <c r="G29" s="9"/>
       <c r="H29" s="7"/>
-      <c r="I29" s="5"/>
-      <c r="J29" s="11"/>
-      <c r="K29" s="12"/>
-      <c r="L29" s="13"/>
-      <c r="M29" s="14"/>
+      <c r="I29" s="7"/>
+      <c r="J29" s="5"/>
+      <c r="K29" s="11"/>
+      <c r="L29" s="12"/>
+      <c r="M29" s="13"/>
       <c r="N29" s="14"/>
-      <c r="O29" s="9"/>
+      <c r="O29" s="14"/>
       <c r="P29" s="9"/>
       <c r="Q29" s="9"/>
       <c r="R29" s="9"/>
       <c r="S29" s="9"/>
-      <c r="T29" s="5"/>
-      <c r="U29" s="15"/>
+      <c r="T29" s="9"/>
+      <c r="U29" s="5"/>
       <c r="V29" s="15"/>
       <c r="W29" s="15"/>
-      <c r="X29" s="16"/>
+      <c r="X29" s="15"/>
       <c r="Y29" s="16"/>
       <c r="Z29" s="16"/>
-      <c r="AA29" s="15"/>
+      <c r="AA29" s="16"/>
       <c r="AB29" s="15"/>
-      <c r="AC29" s="17"/>
+      <c r="AC29" s="15"/>
       <c r="AD29" s="17"/>
-      <c r="AE29" s="15"/>
+      <c r="AE29" s="17"/>
       <c r="AF29" s="15"/>
-      <c r="AG29" s="18"/>
-      <c r="AH29" s="7"/>
-      <c r="AI29" s="9"/>
-      <c r="AJ29" s="15"/>
-      <c r="AK29" s="9"/>
-      <c r="AL29" s="6"/>
-      <c r="AM29" s="15"/>
-      <c r="AN29" s="16"/>
-      <c r="AO29" s="15"/>
-      <c r="AP29" s="16"/>
-      <c r="AQ29" s="26"/>
-      <c r="AR29" s="16"/>
-      <c r="AS29" s="8"/>
+      <c r="AG29" s="15"/>
+      <c r="AH29" s="18"/>
+      <c r="AI29" s="7"/>
+      <c r="AJ29" s="9"/>
+      <c r="AK29" s="15"/>
+      <c r="AL29" s="9"/>
+      <c r="AM29" s="6"/>
+      <c r="AN29" s="15"/>
+      <c r="AO29" s="16"/>
+      <c r="AP29" s="15"/>
+      <c r="AQ29" s="16"/>
+      <c r="AR29" s="26"/>
+      <c r="AS29" s="16"/>
+      <c r="AT29" s="8"/>
     </row>
-    <row r="30" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="30" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A30" s="5"/>
       <c r="B30" s="6"/>
       <c r="C30" s="7"/>
@@ -6430,45 +6488,46 @@
       <c r="F30" s="10"/>
       <c r="G30" s="9"/>
       <c r="H30" s="7"/>
-      <c r="I30" s="5"/>
-      <c r="J30" s="11"/>
-      <c r="K30" s="12"/>
-      <c r="L30" s="13"/>
-      <c r="M30" s="14"/>
+      <c r="I30" s="7"/>
+      <c r="J30" s="5"/>
+      <c r="K30" s="11"/>
+      <c r="L30" s="12"/>
+      <c r="M30" s="13"/>
       <c r="N30" s="14"/>
-      <c r="O30" s="9"/>
+      <c r="O30" s="14"/>
       <c r="P30" s="9"/>
       <c r="Q30" s="9"/>
       <c r="R30" s="9"/>
       <c r="S30" s="9"/>
-      <c r="T30" s="5"/>
-      <c r="U30" s="15"/>
+      <c r="T30" s="9"/>
+      <c r="U30" s="5"/>
       <c r="V30" s="15"/>
       <c r="W30" s="15"/>
-      <c r="X30" s="16"/>
+      <c r="X30" s="15"/>
       <c r="Y30" s="16"/>
       <c r="Z30" s="16"/>
-      <c r="AA30" s="15"/>
+      <c r="AA30" s="16"/>
       <c r="AB30" s="15"/>
-      <c r="AC30" s="17"/>
+      <c r="AC30" s="15"/>
       <c r="AD30" s="17"/>
-      <c r="AE30" s="15"/>
+      <c r="AE30" s="17"/>
       <c r="AF30" s="15"/>
-      <c r="AG30" s="18"/>
-      <c r="AH30" s="7"/>
-      <c r="AI30" s="9"/>
-      <c r="AJ30" s="15"/>
-      <c r="AK30" s="9"/>
-      <c r="AL30" s="6"/>
-      <c r="AM30" s="15"/>
-      <c r="AN30" s="16"/>
-      <c r="AO30" s="15"/>
-      <c r="AP30" s="16"/>
-      <c r="AQ30" s="26"/>
-      <c r="AR30" s="16"/>
-      <c r="AS30" s="8"/>
+      <c r="AG30" s="15"/>
+      <c r="AH30" s="18"/>
+      <c r="AI30" s="7"/>
+      <c r="AJ30" s="9"/>
+      <c r="AK30" s="15"/>
+      <c r="AL30" s="9"/>
+      <c r="AM30" s="6"/>
+      <c r="AN30" s="15"/>
+      <c r="AO30" s="16"/>
+      <c r="AP30" s="15"/>
+      <c r="AQ30" s="16"/>
+      <c r="AR30" s="26"/>
+      <c r="AS30" s="16"/>
+      <c r="AT30" s="8"/>
     </row>
-    <row r="31" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="31" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A31" s="5"/>
       <c r="B31" s="6"/>
       <c r="C31" s="7"/>
@@ -6477,45 +6536,46 @@
       <c r="F31" s="10"/>
       <c r="G31" s="9"/>
       <c r="H31" s="7"/>
-      <c r="I31" s="5"/>
-      <c r="J31" s="11"/>
-      <c r="K31" s="12"/>
-      <c r="L31" s="13"/>
-      <c r="M31" s="14"/>
+      <c r="I31" s="7"/>
+      <c r="J31" s="5"/>
+      <c r="K31" s="11"/>
+      <c r="L31" s="12"/>
+      <c r="M31" s="13"/>
       <c r="N31" s="14"/>
-      <c r="O31" s="9"/>
+      <c r="O31" s="14"/>
       <c r="P31" s="9"/>
       <c r="Q31" s="9"/>
       <c r="R31" s="9"/>
       <c r="S31" s="9"/>
-      <c r="T31" s="5"/>
-      <c r="U31" s="15"/>
+      <c r="T31" s="9"/>
+      <c r="U31" s="5"/>
       <c r="V31" s="15"/>
       <c r="W31" s="15"/>
-      <c r="X31" s="16"/>
+      <c r="X31" s="15"/>
       <c r="Y31" s="16"/>
       <c r="Z31" s="16"/>
-      <c r="AA31" s="15"/>
+      <c r="AA31" s="16"/>
       <c r="AB31" s="15"/>
-      <c r="AC31" s="17"/>
+      <c r="AC31" s="15"/>
       <c r="AD31" s="17"/>
-      <c r="AE31" s="15"/>
+      <c r="AE31" s="17"/>
       <c r="AF31" s="15"/>
-      <c r="AG31" s="18"/>
-      <c r="AH31" s="7"/>
-      <c r="AI31" s="9"/>
-      <c r="AJ31" s="15"/>
-      <c r="AK31" s="9"/>
-      <c r="AL31" s="6"/>
-      <c r="AM31" s="15"/>
-      <c r="AN31" s="16"/>
-      <c r="AO31" s="15"/>
-      <c r="AP31" s="16"/>
-      <c r="AQ31" s="26"/>
-      <c r="AR31" s="16"/>
-      <c r="AS31" s="8"/>
+      <c r="AG31" s="15"/>
+      <c r="AH31" s="18"/>
+      <c r="AI31" s="7"/>
+      <c r="AJ31" s="9"/>
+      <c r="AK31" s="15"/>
+      <c r="AL31" s="9"/>
+      <c r="AM31" s="6"/>
+      <c r="AN31" s="15"/>
+      <c r="AO31" s="16"/>
+      <c r="AP31" s="15"/>
+      <c r="AQ31" s="16"/>
+      <c r="AR31" s="26"/>
+      <c r="AS31" s="16"/>
+      <c r="AT31" s="8"/>
     </row>
-    <row r="32" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="32" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A32" s="5"/>
       <c r="B32" s="6"/>
       <c r="C32" s="7"/>
@@ -6524,45 +6584,46 @@
       <c r="F32" s="10"/>
       <c r="G32" s="9"/>
       <c r="H32" s="7"/>
-      <c r="I32" s="5"/>
-      <c r="J32" s="11"/>
-      <c r="K32" s="12"/>
-      <c r="L32" s="13"/>
-      <c r="M32" s="14"/>
+      <c r="I32" s="7"/>
+      <c r="J32" s="5"/>
+      <c r="K32" s="11"/>
+      <c r="L32" s="12"/>
+      <c r="M32" s="13"/>
       <c r="N32" s="14"/>
-      <c r="O32" s="9"/>
+      <c r="O32" s="14"/>
       <c r="P32" s="9"/>
       <c r="Q32" s="9"/>
       <c r="R32" s="9"/>
       <c r="S32" s="9"/>
-      <c r="T32" s="5"/>
-      <c r="U32" s="15"/>
+      <c r="T32" s="9"/>
+      <c r="U32" s="5"/>
       <c r="V32" s="15"/>
       <c r="W32" s="15"/>
-      <c r="X32" s="16"/>
+      <c r="X32" s="15"/>
       <c r="Y32" s="16"/>
       <c r="Z32" s="16"/>
-      <c r="AA32" s="15"/>
+      <c r="AA32" s="16"/>
       <c r="AB32" s="15"/>
-      <c r="AC32" s="17"/>
+      <c r="AC32" s="15"/>
       <c r="AD32" s="17"/>
-      <c r="AE32" s="15"/>
+      <c r="AE32" s="17"/>
       <c r="AF32" s="15"/>
-      <c r="AG32" s="18"/>
-      <c r="AH32" s="7"/>
-      <c r="AI32" s="9"/>
-      <c r="AJ32" s="15"/>
-      <c r="AK32" s="9"/>
-      <c r="AL32" s="6"/>
-      <c r="AM32" s="15"/>
-      <c r="AN32" s="16"/>
-      <c r="AO32" s="15"/>
-      <c r="AP32" s="16"/>
-      <c r="AQ32" s="26"/>
-      <c r="AR32" s="16"/>
-      <c r="AS32" s="8"/>
+      <c r="AG32" s="15"/>
+      <c r="AH32" s="18"/>
+      <c r="AI32" s="7"/>
+      <c r="AJ32" s="9"/>
+      <c r="AK32" s="15"/>
+      <c r="AL32" s="9"/>
+      <c r="AM32" s="6"/>
+      <c r="AN32" s="15"/>
+      <c r="AO32" s="16"/>
+      <c r="AP32" s="15"/>
+      <c r="AQ32" s="16"/>
+      <c r="AR32" s="26"/>
+      <c r="AS32" s="16"/>
+      <c r="AT32" s="8"/>
     </row>
-    <row r="33" spans="1:45" ht="17" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="33" spans="1:46" ht="17" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A33" s="5"/>
       <c r="B33" s="6"/>
       <c r="C33" s="7"/>
@@ -6571,43 +6632,44 @@
       <c r="F33" s="10"/>
       <c r="G33" s="9"/>
       <c r="H33" s="7"/>
-      <c r="I33" s="5"/>
-      <c r="J33" s="11"/>
-      <c r="K33" s="12"/>
-      <c r="L33" s="13"/>
-      <c r="M33" s="14"/>
+      <c r="I33" s="7"/>
+      <c r="J33" s="5"/>
+      <c r="K33" s="11"/>
+      <c r="L33" s="12"/>
+      <c r="M33" s="13"/>
       <c r="N33" s="14"/>
-      <c r="O33" s="9"/>
+      <c r="O33" s="14"/>
       <c r="P33" s="9"/>
       <c r="Q33" s="9"/>
       <c r="R33" s="9"/>
       <c r="S33" s="9"/>
-      <c r="T33" s="5"/>
-      <c r="U33" s="15"/>
+      <c r="T33" s="9"/>
+      <c r="U33" s="5"/>
       <c r="V33" s="15"/>
       <c r="W33" s="15"/>
-      <c r="X33" s="16"/>
+      <c r="X33" s="15"/>
       <c r="Y33" s="16"/>
       <c r="Z33" s="16"/>
-      <c r="AA33" s="15"/>
+      <c r="AA33" s="16"/>
       <c r="AB33" s="15"/>
-      <c r="AC33" s="17"/>
+      <c r="AC33" s="15"/>
       <c r="AD33" s="17"/>
-      <c r="AE33" s="15"/>
+      <c r="AE33" s="17"/>
       <c r="AF33" s="15"/>
-      <c r="AG33" s="18"/>
-      <c r="AH33" s="7"/>
-      <c r="AI33" s="9"/>
-      <c r="AJ33" s="15"/>
-      <c r="AK33" s="9"/>
-      <c r="AL33" s="6"/>
-      <c r="AM33" s="15"/>
-      <c r="AN33" s="16"/>
-      <c r="AO33" s="15"/>
-      <c r="AP33" s="16"/>
-      <c r="AQ33" s="26"/>
-      <c r="AR33" s="16"/>
-      <c r="AS33" s="8"/>
+      <c r="AG33" s="15"/>
+      <c r="AH33" s="18"/>
+      <c r="AI33" s="7"/>
+      <c r="AJ33" s="9"/>
+      <c r="AK33" s="15"/>
+      <c r="AL33" s="9"/>
+      <c r="AM33" s="6"/>
+      <c r="AN33" s="15"/>
+      <c r="AO33" s="16"/>
+      <c r="AP33" s="15"/>
+      <c r="AQ33" s="16"/>
+      <c r="AR33" s="26"/>
+      <c r="AS33" s="16"/>
+      <c r="AT33" s="8"/>
     </row>
   </sheetData>
   <phoneticPr fontId="9" type="noConversion"/>

</xml_diff>